<commit_message>
Add market growth notes and extend cost model with market slides
Two working notes estimate the proton-therapy installed base for 2036
and 2046 from PTCOG lists, IBA investor reports and demand bounds.
The cost model gains market_growth and argos_market tables, the deck
now includes six generated economics slides, and LaTeX build
artifacts are ignored.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LunF6tV69q7Y6sP6GhwFZb
</commit_message>
<xml_diff>
--- a/costs/costs.xlsx
+++ b/costs/costs.xlsx
@@ -11,13 +11,15 @@
     <sheet name="installation_market" sheetId="2" r:id="rId2"/>
     <sheet name="annual_service" sheetId="3" r:id="rId3"/>
     <sheet name="recurring_market" sheetId="4" r:id="rId4"/>
+    <sheet name="market_growth" sheetId="5" r:id="rId5"/>
+    <sheet name="argos_market" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="350">
   <si>
     <t>ID</t>
   </si>
@@ -115,7 +117,7 @@
     <t>fraction</t>
   </si>
   <si>
-    <t>Planning target, not an industry benchmark.</t>
+    <t>Historical 40% pricing reference; current commercial price is an independent input.</t>
   </si>
   <si>
     <t>installation_target_price</t>
@@ -130,7 +132,7 @@
     <t>installation_price</t>
   </si>
   <si>
-    <t>Agreed selling ticket</t>
+    <t>Installed system price</t>
   </si>
   <si>
     <t>Excludes VAT; includes initial software licence and standard commissioning.</t>
@@ -178,6 +180,24 @@
     <t>installation_example_count*installation_price</t>
   </si>
   <si>
+    <t>installation_negotiated_price</t>
+  </si>
+  <si>
+    <t>Negotiated system price scenario</t>
+  </si>
+  <si>
+    <t>Price sensitivity; not the target commercial offer.</t>
+  </si>
+  <si>
+    <t>installation_negotiated_margin</t>
+  </si>
+  <si>
+    <t>Negotiated system gross margin</t>
+  </si>
+  <si>
+    <t>(installation_negotiated_price-delivered_cost)/installation_negotiated_price</t>
+  </si>
+  <si>
     <t>room_order_year</t>
   </si>
   <si>
@@ -544,9 +564,6 @@
     <t>Target service gross margin</t>
   </si>
   <si>
-    <t>Planning target.</t>
-  </si>
-  <si>
     <t>service_target_price</t>
   </si>
   <si>
@@ -559,7 +576,7 @@
     <t>service_price</t>
   </si>
   <si>
-    <t>Agreed annual service ticket</t>
+    <t>Annual service fee</t>
   </si>
   <si>
     <t>Accepted by user; excludes VAT. Service after included installation warranty; avoid charging twice for warranty coverage.</t>
@@ -586,6 +603,36 @@
     <t>service_profit/service_price</t>
   </si>
   <si>
+    <t>service_price_ratio</t>
+  </si>
+  <si>
+    <t>Annual fee as share of system selling price</t>
+  </si>
+  <si>
+    <t>service_price/installation_price</t>
+  </si>
+  <si>
+    <t>Comparison with selling price, not manufacturing cost.</t>
+  </si>
+  <si>
+    <t>service_negotiated_price</t>
+  </si>
+  <si>
+    <t>Negotiated annual service fee scenario</t>
+  </si>
+  <si>
+    <t>Price sensitivity; agreed scope unchanged.</t>
+  </si>
+  <si>
+    <t>service_negotiated_margin</t>
+  </si>
+  <si>
+    <t>Negotiated service gross margin</t>
+  </si>
+  <si>
+    <t>(service_negotiated_price-service_cost)/service_negotiated_price</t>
+  </si>
+  <si>
     <t>recurring_price</t>
   </si>
   <si>
@@ -710,6 +757,318 @@
   </si>
   <si>
     <t>large_contracts*recurring_profit</t>
+  </si>
+  <si>
+    <t>growth_start_year</t>
+  </si>
+  <si>
+    <t>Reference year</t>
+  </si>
+  <si>
+    <t>growth_base</t>
+  </si>
+  <si>
+    <t>Provisional operating proton rooms</t>
+  </si>
+  <si>
+    <t>Planning assumption; not a verified inventory or ARGOS-compatible base.</t>
+  </si>
+  <si>
+    <t>growth_short</t>
+  </si>
+  <si>
+    <t>First horizon</t>
+  </si>
+  <si>
+    <t>years</t>
+  </si>
+  <si>
+    <t>growth_long</t>
+  </si>
+  <si>
+    <t>Second horizon</t>
+  </si>
+  <si>
+    <t>growth_short_year</t>
+  </si>
+  <si>
+    <t>First projection year</t>
+  </si>
+  <si>
+    <t>growth_start_year+growth_short</t>
+  </si>
+  <si>
+    <t>growth_long_year</t>
+  </si>
+  <si>
+    <t>Second projection year</t>
+  </si>
+  <si>
+    <t>growth_start_year+growth_long</t>
+  </si>
+  <si>
+    <t>growth_slow</t>
+  </si>
+  <si>
+    <t>Assumed annual net growth: slow</t>
+  </si>
+  <si>
+    <t>Judgement-based scenario; not a fitted forecast or confidence interval.</t>
+  </si>
+  <si>
+    <t>slow_short</t>
+  </si>
+  <si>
+    <t>Operating rooms: slow short</t>
+  </si>
+  <si>
+    <t>growth_base*(1+growth_slow)**growth_short</t>
+  </si>
+  <si>
+    <t>slow_short_shown</t>
+  </si>
+  <si>
+    <t>Rounded rooms: slow short</t>
+  </si>
+  <si>
+    <t>round(slow_short,0)</t>
+  </si>
+  <si>
+    <t>slow_long</t>
+  </si>
+  <si>
+    <t>Operating rooms: slow long</t>
+  </si>
+  <si>
+    <t>growth_base*(1+growth_slow)**growth_long</t>
+  </si>
+  <si>
+    <t>slow_long_shown</t>
+  </si>
+  <si>
+    <t>Rounded rooms: slow long</t>
+  </si>
+  <si>
+    <t>round(slow_long,0)</t>
+  </si>
+  <si>
+    <t>growth_central</t>
+  </si>
+  <si>
+    <t>Assumed annual net growth: central</t>
+  </si>
+  <si>
+    <t>central_short</t>
+  </si>
+  <si>
+    <t>Operating rooms: central short</t>
+  </si>
+  <si>
+    <t>growth_base*(1+growth_central)**growth_short</t>
+  </si>
+  <si>
+    <t>central_short_shown</t>
+  </si>
+  <si>
+    <t>Rounded rooms: central short</t>
+  </si>
+  <si>
+    <t>round(central_short,0)</t>
+  </si>
+  <si>
+    <t>central_long</t>
+  </si>
+  <si>
+    <t>Operating rooms: central long</t>
+  </si>
+  <si>
+    <t>growth_base*(1+growth_central)**growth_long</t>
+  </si>
+  <si>
+    <t>central_long_shown</t>
+  </si>
+  <si>
+    <t>Rounded rooms: central long</t>
+  </si>
+  <si>
+    <t>round(central_long,0)</t>
+  </si>
+  <si>
+    <t>growth_fast</t>
+  </si>
+  <si>
+    <t>Assumed annual net growth: fast</t>
+  </si>
+  <si>
+    <t>fast_short</t>
+  </si>
+  <si>
+    <t>Operating rooms: fast short</t>
+  </si>
+  <si>
+    <t>growth_base*(1+growth_fast)**growth_short</t>
+  </si>
+  <si>
+    <t>fast_short_shown</t>
+  </si>
+  <si>
+    <t>Rounded rooms: fast short</t>
+  </si>
+  <si>
+    <t>round(fast_short,0)</t>
+  </si>
+  <si>
+    <t>fast_long</t>
+  </si>
+  <si>
+    <t>Operating rooms: fast long</t>
+  </si>
+  <si>
+    <t>growth_base*(1+growth_fast)**growth_long</t>
+  </si>
+  <si>
+    <t>fast_long_shown</t>
+  </si>
+  <si>
+    <t>Rounded rooms: fast long</t>
+  </si>
+  <si>
+    <t>round(fast_long,0)</t>
+  </si>
+  <si>
+    <t>observed_centres</t>
+  </si>
+  <si>
+    <t>Proton facilities January 2026</t>
+  </si>
+  <si>
+    <t>centres</t>
+  </si>
+  <si>
+    <t>Yap et al. doi:10.3389/fonc.2026.1791102; PTCOG compilation.</t>
+  </si>
+  <si>
+    <t>construction_rooms</t>
+  </si>
+  <si>
+    <t>Listed proton rooms under construction June 2026</t>
+  </si>
+  <si>
+    <t>Manual PTCOG tally; includes stale/uncertain dates; excludes carbon-only rooms. https://ptcog.online/facilities-under-construction/</t>
+  </si>
+  <si>
+    <t>recent_iba_orders</t>
+  </si>
+  <si>
+    <t>IBA H1 2026 room orders</t>
+  </si>
+  <si>
+    <t>IBA H1 2026 presentation p13.</t>
+  </si>
+  <si>
+    <t>recent_iba_share</t>
+  </si>
+  <si>
+    <t>IBA H1 2026 reported order share</t>
+  </si>
+  <si>
+    <t>https://www.iba-worldwide.com/sites/default/files/2026-08/iba_h1_2026_results_presentation.pdf</t>
+  </si>
+  <si>
+    <t>recent_global_orders</t>
+  </si>
+  <si>
+    <t>Implied H1 global room orders</t>
+  </si>
+  <si>
+    <t>round(recent_iba_orders/recent_iba_share,0)</t>
+  </si>
+  <si>
+    <t>recent_iba_backlog</t>
+  </si>
+  <si>
+    <t>IBA H1 2026 equipment projects</t>
+  </si>
+  <si>
+    <t>projects</t>
+  </si>
+  <si>
+    <t>7 ProteusPLUS and 39 ProteusONE; includes 11 installations underway. Overlaps PTCOG pipeline.</t>
+  </si>
+  <si>
+    <t>tam_price</t>
+  </si>
+  <si>
+    <t>Price per ARGOS system</t>
+  </si>
+  <si>
+    <t>tam_fee</t>
+  </si>
+  <si>
+    <t>tam_short_added</t>
+  </si>
+  <si>
+    <t>Cumulative net additional rooms</t>
+  </si>
+  <si>
+    <t>central_short-growth_base</t>
+  </si>
+  <si>
+    <t>tam_short_added_shown</t>
+  </si>
+  <si>
+    <t>Rounded cumulative net additional rooms</t>
+  </si>
+  <si>
+    <t>round(tam_short_added,0)</t>
+  </si>
+  <si>
+    <t>tam_short_systems</t>
+  </si>
+  <si>
+    <t>Cumulative system sales potential from net expansion</t>
+  </si>
+  <si>
+    <t>tam_short_added*tam_price</t>
+  </si>
+  <si>
+    <t>Full compatibility and adoption; all suppliers; excludes existing-base retrofits and replacement. Uses unrounded projections.</t>
+  </si>
+  <si>
+    <t>tam_short_services</t>
+  </si>
+  <si>
+    <t>Annual service potential on entire projected room base</t>
+  </si>
+  <si>
+    <t>central_short*tam_fee</t>
+  </si>
+  <si>
+    <t>Full compatibility and adoption; all projected operating rooms on full-year contracts. All suppliers, not ARGOS company revenue.</t>
+  </si>
+  <si>
+    <t>tam_long_added</t>
+  </si>
+  <si>
+    <t>central_long-growth_base</t>
+  </si>
+  <si>
+    <t>tam_long_added_shown</t>
+  </si>
+  <si>
+    <t>round(tam_long_added,0)</t>
+  </si>
+  <si>
+    <t>tam_long_systems</t>
+  </si>
+  <si>
+    <t>tam_long_added*tam_price</t>
+  </si>
+  <si>
+    <t>tam_long_services</t>
+  </si>
+  <si>
+    <t>central_long*tam_fee</t>
   </si>
 </sst>
 </file>
@@ -773,8 +1132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="model_installation" displayName="model_installation" ref="A1:G14" totalsRowShown="0">
-  <autoFilter ref="A1:G14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="model_installation" displayName="model_installation" ref="A1:G16" totalsRowShown="0">
+  <autoFilter ref="A1:G16"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -805,8 +1164,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="model_annual_service" displayName="model_annual_service" ref="A1:G27" totalsRowShown="0">
-  <autoFilter ref="A1:G27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="model_annual_service" displayName="model_annual_service" ref="A1:G30" totalsRowShown="0">
+  <autoFilter ref="A1:G30"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -823,6 +1182,38 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="model_recurring_market" displayName="model_recurring_market" ref="A1:G16" totalsRowShown="0">
   <autoFilter ref="A1:G16"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Item"/>
+    <tableColumn id="3" name="Kind"/>
+    <tableColumn id="4" name="Value"/>
+    <tableColumn id="5" name="Unit"/>
+    <tableColumn id="6" name="Calculation"/>
+    <tableColumn id="7" name="Assumption / source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="model_market_growth" displayName="model_market_growth" ref="A1:G28" totalsRowShown="0">
+  <autoFilter ref="A1:G28"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Item"/>
+    <tableColumn id="3" name="Kind"/>
+    <tableColumn id="4" name="Value"/>
+    <tableColumn id="5" name="Unit"/>
+    <tableColumn id="6" name="Calculation"/>
+    <tableColumn id="7" name="Assumption / source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="model_argos_market" displayName="model_argos_market" ref="A1:G11" totalsRowShown="0">
+  <autoFilter ref="A1:G11"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -1121,7 +1512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1251,7 +1642,7 @@
         <v>9</v>
       </c>
       <c r="D6" s="1">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -1272,7 +1663,7 @@
       </c>
       <c r="D7" s="2">
         <f>('installation'!D4+'installation'!D6)</f>
-        <v>1300000.0</v>
+        <v>1200000.0</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -1313,7 +1704,7 @@
       </c>
       <c r="D9" s="2">
         <f>('installation'!D7/(1-'installation'!D8))</f>
-        <v>2166666.666666667</v>
+        <v>2000000.0</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1333,7 +1724,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="1">
-        <v>2200000</v>
+        <v>2500000</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1354,7 +1745,7 @@
       </c>
       <c r="D11" s="2">
         <f>('installation'!D10-'installation'!D7)</f>
-        <v>900000.0</v>
+        <v>1300000.0</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1378,7 +1769,7 @@
       </c>
       <c r="D12" s="4">
         <f>('installation'!D11/'installation'!D10)</f>
-        <v>0.4090909090909091</v>
+        <v>0.52</v>
       </c>
       <c r="E12" t="s">
         <v>31</v>
@@ -1419,13 +1810,54 @@
       </c>
       <c r="D14" s="2">
         <f>('installation'!D13*'installation'!D10)</f>
-        <v>22000000.0</v>
+        <v>25000000.0</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
       </c>
       <c r="F14" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2200000</v>
+      </c>
+      <c r="E15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="4">
+        <f>(('installation'!D15-'installation'!D7)/'installation'!D15)</f>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="E16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1475,10 +1907,10 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -1487,18 +1919,18 @@
         <v>2025</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -1507,18 +1939,18 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G3" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1530,15 +1962,15 @@
         <v>31</v>
       </c>
       <c r="G4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -1548,18 +1980,18 @@
         <v>19.047619047619047</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F5" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
@@ -1569,21 +2001,21 @@
         <v>19.0</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -1595,15 +2027,15 @@
         <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -1613,25 +2045,25 @@
         <v>19.0</v>
       </c>
       <c r="E8" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="2">
         <f>'installation'!D10</f>
-        <v>2200000.0</v>
+        <v>2500000.0</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1642,31 +2074,31 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2">
         <f>('installation_market'!D8*'installation_market'!D9)</f>
-        <v>41800000.0</v>
+        <v>47500000.0</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -1675,18 +2107,18 @@
         <v>300</v>
       </c>
       <c r="E11" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="G11" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
         <v>9</v>
@@ -1698,15 +2130,15 @@
         <v>31</v>
       </c>
       <c r="G12" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -1716,39 +2148,39 @@
         <v>15.0</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F13" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="2">
         <f>('installation_market'!D13*'installation_market'!D9)</f>
-        <v>33000000.0</v>
+        <v>37500000.0</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B15" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -1758,58 +2190,58 @@
         <v>34.0</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F15" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="2">
         <f>('installation_market'!D10+'installation_market'!D14)</f>
-        <v>74800000.0</v>
+        <v>85000000.0</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G16" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
       </c>
       <c r="D17" s="2">
         <f>('installation_market'!D11*'installation_market'!D9)</f>
-        <v>660000000.0</v>
+        <v>750000000.0</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1822,7 +2254,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1859,10 +2291,10 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -1871,18 +2303,18 @@
         <v>8000</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -1891,18 +2323,18 @@
         <v>10000</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1911,18 +2343,18 @@
         <v>7000</v>
       </c>
       <c r="E4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G4" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -1931,18 +2363,18 @@
         <v>5000</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
@@ -1952,21 +2384,21 @@
         <v>30000.0</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -1975,18 +2407,18 @@
         <v>50000</v>
       </c>
       <c r="E7" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G7" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B8" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C8" t="s">
         <v>9</v>
@@ -1998,15 +2430,15 @@
         <v>31</v>
       </c>
       <c r="G8" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B9" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
@@ -2016,18 +2448,18 @@
         <v>16000.0</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F9" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
@@ -2037,18 +2469,18 @@
         <v>66000.0</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F10" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -2060,15 +2492,15 @@
         <v>31</v>
       </c>
       <c r="G11" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
@@ -2078,18 +2510,18 @@
         <v>13200.0</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -2099,18 +2531,18 @@
         <v>79200.0</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B14" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="C14" t="s">
         <v>9</v>
@@ -2122,15 +2554,15 @@
         <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -2140,18 +2572,18 @@
         <v>80000.0</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B16" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C16" t="s">
         <v>9</v>
@@ -2160,18 +2592,18 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="G16" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B17" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -2181,18 +2613,18 @@
         <v>80000.0</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F17" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B18" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C18" t="s">
         <v>9</v>
@@ -2201,18 +2633,18 @@
         <v>2000</v>
       </c>
       <c r="E18" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G18" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B19" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C19" t="s">
         <v>9</v>
@@ -2221,18 +2653,18 @@
         <v>1000</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G19" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B20" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C20" t="s">
         <v>9</v>
@@ -2241,18 +2673,18 @@
         <v>2000</v>
       </c>
       <c r="E20" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G20" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B21" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C21" t="s">
         <v>20</v>
@@ -2262,21 +2694,21 @@
         <v>5000.0</v>
       </c>
       <c r="E21" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F21" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="G21" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B22" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C22" t="s">
         <v>20</v>
@@ -2286,18 +2718,18 @@
         <v>115000.0</v>
       </c>
       <c r="E22" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F22" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B23" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
@@ -2309,15 +2741,15 @@
         <v>31</v>
       </c>
       <c r="G23" t="s">
-        <v>175</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B24" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C24" t="s">
         <v>20</v>
@@ -2327,75 +2759,140 @@
         <v>191666.6666666667</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F24" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C25" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="1">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="E25" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G25" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B26" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C26" t="s">
         <v>20</v>
       </c>
       <c r="D26" s="2">
         <f>('annual_service'!D25-'annual_service'!D22)</f>
-        <v>85000.0</v>
+        <v>135000.0</v>
       </c>
       <c r="E26" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="G26" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B27" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C27" t="s">
         <v>20</v>
       </c>
       <c r="D27" s="4">
         <f>('annual_service'!D26/'annual_service'!D25)</f>
-        <v>0.425</v>
+        <v>0.54</v>
       </c>
       <c r="E27" t="s">
         <v>31</v>
       </c>
       <c r="F27" t="s">
-        <v>188</v>
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>194</v>
+      </c>
+      <c r="B28" t="s">
+        <v>195</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" s="4">
+        <f>('annual_service'!D25/'installation'!D10)</f>
+        <v>0.1</v>
+      </c>
+      <c r="E28" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" t="s">
+        <v>196</v>
+      </c>
+      <c r="G28" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>198</v>
+      </c>
+      <c r="B29" t="s">
+        <v>199</v>
+      </c>
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="1">
+        <v>200000</v>
+      </c>
+      <c r="E29" t="s">
+        <v>87</v>
+      </c>
+      <c r="G29" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30" t="s">
+        <v>202</v>
+      </c>
+      <c r="C30" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="4">
+        <f>(('annual_service'!D29-'annual_service'!D22)/'annual_service'!D29)</f>
+        <v>0.425</v>
+      </c>
+      <c r="E30" t="s">
+        <v>31</v>
+      </c>
+      <c r="F30" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2445,31 +2942,31 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="B2" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
       </c>
       <c r="D2" s="2">
         <f>'annual_service'!D25</f>
-        <v>200000.0</v>
+        <v>250000.0</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="B3" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -2479,39 +2976,39 @@
         <v>115000.0</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="B4" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="2">
         <f>'annual_service'!D26</f>
-        <v>85000.0</v>
+        <v>135000.0</v>
       </c>
       <c r="E4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F4" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="B5" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -2520,39 +3017,39 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="G5" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="B6" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" s="2">
         <f>('recurring_market'!D5*'recurring_market'!D2)</f>
-        <v>2000000.0</v>
+        <v>2500000.0</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="B7" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -2562,42 +3059,42 @@
         <v>1150000.0</v>
       </c>
       <c r="E7" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F7" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="B8" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="2">
         <f>('recurring_market'!D5*'recurring_market'!D4)</f>
-        <v>850000.0</v>
+        <v>1350000.0</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F8" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="G8" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="B9" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="C9" t="s">
         <v>9</v>
@@ -2606,39 +3103,39 @@
         <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="G9" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="B10" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2">
         <f>('recurring_market'!D9*'recurring_market'!D2)</f>
-        <v>20000000.0</v>
+        <v>25000000.0</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F10" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="B11" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
@@ -2648,42 +3145,42 @@
         <v>11500000.0</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F11" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="B12" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
       </c>
       <c r="D12" s="2">
         <f>('recurring_market'!D9*'recurring_market'!D4)</f>
-        <v>8500000.0</v>
+        <v>13500000.0</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
       <c r="G12" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="B13" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
@@ -2692,39 +3189,39 @@
         <v>300</v>
       </c>
       <c r="E13" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="G13" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="B14" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="2">
         <f>('recurring_market'!D13*'recurring_market'!D2)</f>
-        <v>60000000.0</v>
+        <v>75000000.0</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="B15" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -2734,34 +3231,892 @@
         <v>34500000.0</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="B16" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="2">
         <f>('recurring_market'!D13*'recurring_market'!D4)</f>
-        <v>25500000.0</v>
+        <v>40500000.0</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="G16" t="s">
-        <v>208</v>
+        <v>223</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="57.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="57.7109375" customWidth="1"/>
+    <col min="7" max="7" width="100.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2026</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1">
+        <v>300</v>
+      </c>
+      <c r="E3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B4" t="s">
+        <v>252</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>256</v>
+      </c>
+      <c r="B6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <f>('market_growth'!D2+'market_growth'!D4)</f>
+        <v>2036.0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>259</v>
+      </c>
+      <c r="B7" t="s">
+        <v>260</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <f>('market_growth'!D2+'market_growth'!D5)</f>
+        <v>2046.0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B8" t="s">
+        <v>263</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>265</v>
+      </c>
+      <c r="B9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <f>('market_growth'!D3*((1+'market_growth'!D8)^'market_growth'!D4))</f>
+        <v>403.1749138032367</v>
+      </c>
+      <c r="E9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F9" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>268</v>
+      </c>
+      <c r="B10" t="s">
+        <v>269</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="2">
+        <f>ROUND('market_growth'!D9,0)</f>
+        <v>403.0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F10" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2">
+        <f>('market_growth'!D3*((1+'market_growth'!D8)^'market_growth'!D5))</f>
+        <v>541.8333704008245</v>
+      </c>
+      <c r="E11" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>274</v>
+      </c>
+      <c r="B12" t="s">
+        <v>275</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2">
+        <f>ROUND('market_growth'!D11,0)</f>
+        <v>542.0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>277</v>
+      </c>
+      <c r="B13" t="s">
+        <v>278</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>279</v>
+      </c>
+      <c r="B14" t="s">
+        <v>280</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2">
+        <f>('market_growth'!D3*((1+'market_growth'!D13)^'market_growth'!D4))</f>
+        <v>488.6683880332326</v>
+      </c>
+      <c r="E14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>282</v>
+      </c>
+      <c r="B15" t="s">
+        <v>283</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="2">
+        <f>ROUND('market_growth'!D14,0)</f>
+        <v>489.0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>285</v>
+      </c>
+      <c r="B16" t="s">
+        <v>286</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2">
+        <f>('market_growth'!D3*((1+'market_growth'!D13)^'market_growth'!D5))</f>
+        <v>795.9893115433266</v>
+      </c>
+      <c r="E16" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>288</v>
+      </c>
+      <c r="B17" t="s">
+        <v>289</v>
+      </c>
+      <c r="C17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2">
+        <f>ROUND('market_growth'!D16,0)</f>
+        <v>796.0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>291</v>
+      </c>
+      <c r="B18" t="s">
+        <v>292</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>293</v>
+      </c>
+      <c r="B19" t="s">
+        <v>294</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="2">
+        <f>('market_growth'!D3*((1+'market_growth'!D18)^'market_growth'!D4))</f>
+        <v>590.14540718687</v>
+      </c>
+      <c r="E19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>296</v>
+      </c>
+      <c r="B20" t="s">
+        <v>297</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="2">
+        <f>ROUND('market_growth'!D19,0)</f>
+        <v>590.0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>299</v>
+      </c>
+      <c r="B21" t="s">
+        <v>300</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="2">
+        <f>('market_growth'!D3*((1+'market_growth'!D18)^'market_growth'!D5))</f>
+        <v>1160.905338745855</v>
+      </c>
+      <c r="E21" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>302</v>
+      </c>
+      <c r="B22" t="s">
+        <v>303</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="2">
+        <f>ROUND('market_growth'!D21,0)</f>
+        <v>1161.0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>305</v>
+      </c>
+      <c r="B23" t="s">
+        <v>306</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="1">
+        <v>128</v>
+      </c>
+      <c r="E23" t="s">
+        <v>307</v>
+      </c>
+      <c r="G23" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>309</v>
+      </c>
+      <c r="B24" t="s">
+        <v>310</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="1">
+        <v>57</v>
+      </c>
+      <c r="E24" t="s">
+        <v>91</v>
+      </c>
+      <c r="G24" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>312</v>
+      </c>
+      <c r="B25" t="s">
+        <v>313</v>
+      </c>
+      <c r="C25" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="1">
+        <v>5</v>
+      </c>
+      <c r="E25" t="s">
+        <v>91</v>
+      </c>
+      <c r="G25" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>315</v>
+      </c>
+      <c r="B26" t="s">
+        <v>316</v>
+      </c>
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.31</v>
+      </c>
+      <c r="E26" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>318</v>
+      </c>
+      <c r="B27" t="s">
+        <v>319</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" s="2">
+        <f>ROUND(('market_growth'!D25/'market_growth'!D26),0)</f>
+        <v>16.0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>91</v>
+      </c>
+      <c r="F27" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>321</v>
+      </c>
+      <c r="B28" t="s">
+        <v>322</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="1">
+        <v>46</v>
+      </c>
+      <c r="E28" t="s">
+        <v>323</v>
+      </c>
+      <c r="G28" t="s">
+        <v>324</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="57.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="57.7109375" customWidth="1"/>
+    <col min="7" max="7" width="100.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2">
+        <f>'installation'!D10</f>
+        <v>2500000.0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2">
+        <f>'annual_service'!D25</f>
+        <v>250000.0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B4" t="s">
+        <v>329</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2">
+        <f>('market_growth'!D14-'market_growth'!D3)</f>
+        <v>188.6683880332326</v>
+      </c>
+      <c r="E4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>331</v>
+      </c>
+      <c r="B5" t="s">
+        <v>332</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2">
+        <f>ROUND('argos_market'!D4,0)</f>
+        <v>189.0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>334</v>
+      </c>
+      <c r="B6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <f>('argos_market'!D4*'argos_market'!D2)</f>
+        <v>471670970.0830815</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>336</v>
+      </c>
+      <c r="G6" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B7" t="s">
+        <v>339</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <f>('market_growth'!D14*'argos_market'!D3)</f>
+        <v>122167097.00830814</v>
+      </c>
+      <c r="E7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" t="s">
+        <v>340</v>
+      </c>
+      <c r="G7" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>342</v>
+      </c>
+      <c r="B8" t="s">
+        <v>329</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2">
+        <f>('market_growth'!D16-'market_growth'!D3)</f>
+        <v>495.9893115433266</v>
+      </c>
+      <c r="E8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>344</v>
+      </c>
+      <c r="B9" t="s">
+        <v>332</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <f>ROUND('argos_market'!D8,0)</f>
+        <v>496.0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F9" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>346</v>
+      </c>
+      <c r="B10" t="s">
+        <v>335</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="2">
+        <f>('argos_market'!D8*'argos_market'!D2)</f>
+        <v>1239973278.8583164</v>
+      </c>
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>347</v>
+      </c>
+      <c r="G10" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>348</v>
+      </c>
+      <c r="B11" t="s">
+        <v>339</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2">
+        <f>('market_growth'!D16*'argos_market'!D3)</f>
+        <v>198997327.88583165</v>
+      </c>
+      <c r="E11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" t="s">
+        <v>349</v>
+      </c>
+      <c r="G11" t="s">
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add four-year startup budget and EUR 4M funding slides
</commit_message>
<xml_diff>
--- a/costs/costs.xlsx
+++ b/costs/costs.xlsx
@@ -13,13 +13,16 @@
     <sheet name="recurring_market" sheetId="4" r:id="rId4"/>
     <sheet name="market_growth" sheetId="5" r:id="rId5"/>
     <sheet name="argos_market" sheetId="6" r:id="rId6"/>
+    <sheet name="costs-reduced" sheetId="7" r:id="rId7"/>
+    <sheet name="startup_team" sheetId="8" r:id="rId8"/>
+    <sheet name="startup_programme" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="586">
   <si>
     <t>ID</t>
   </si>
@@ -1069,6 +1072,714 @@
   </si>
   <si>
     <t>central_long*tam_fee</t>
+  </si>
+  <si>
+    <t>startup_years</t>
+  </si>
+  <si>
+    <t>Programme duration</t>
+  </si>
+  <si>
+    <t>startup_pet</t>
+  </si>
+  <si>
+    <t>startup_camera</t>
+  </si>
+  <si>
+    <t>startup_other_hardware</t>
+  </si>
+  <si>
+    <t>Computing and other hardware</t>
+  </si>
+  <si>
+    <t>User input for independent reduced estimate.</t>
+  </si>
+  <si>
+    <t>startup_raw</t>
+  </si>
+  <si>
+    <t>Raw hardware total</t>
+  </si>
+  <si>
+    <t>startup_pet+startup_camera+startup_other_hardware</t>
+  </si>
+  <si>
+    <t>startup_external_work</t>
+  </si>
+  <si>
+    <t>Prototype fabrication and test equipment</t>
+  </si>
+  <si>
+    <t>External purchases and contracted work only; employee labour is in personnel.</t>
+  </si>
+  <si>
+    <t>startup_device_reserve</t>
+  </si>
+  <si>
+    <t>First-device contingency</t>
+  </si>
+  <si>
+    <t>Fixed EUR 300000 first-device contingency; user revision.</t>
+  </si>
+  <si>
+    <t>startup_hardware_package</t>
+  </si>
+  <si>
+    <t>Hardware and prototype package including contingency</t>
+  </si>
+  <si>
+    <t>startup_raw+startup_external_work+startup_device_reserve</t>
+  </si>
+  <si>
+    <t>startup_ceo_fte</t>
+  </si>
+  <si>
+    <t>CEO / project and business lead: staffing</t>
+  </si>
+  <si>
+    <t>FTE</t>
+  </si>
+  <si>
+    <t>startup_ceo_annual</t>
+  </si>
+  <si>
+    <t>CEO / project and business lead: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>startup_ceo_years</t>
+  </si>
+  <si>
+    <t>CEO / project and business lead: funded years</t>
+  </si>
+  <si>
+    <t>startup_ceo_total</t>
+  </si>
+  <si>
+    <t>CEO / project and business lead: programme cost</t>
+  </si>
+  <si>
+    <t>startup_ceo_fte*startup_ceo_annual*startup_ceo_years</t>
+  </si>
+  <si>
+    <t>startup_architect_fte</t>
+  </si>
+  <si>
+    <t>System architect / technical lead: staffing</t>
+  </si>
+  <si>
+    <t>Lead architect removed by user; zero retained for editable formulas.</t>
+  </si>
+  <si>
+    <t>startup_architect_annual</t>
+  </si>
+  <si>
+    <t>System architect / technical lead: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>Includes employer contributions.</t>
+  </si>
+  <si>
+    <t>startup_architect_years</t>
+  </si>
+  <si>
+    <t>System architect / technical lead: funded years</t>
+  </si>
+  <si>
+    <t>startup_architect_total</t>
+  </si>
+  <si>
+    <t>System architect / technical lead: programme cost</t>
+  </si>
+  <si>
+    <t>startup_architect_fte*startup_architect_annual*startup_architect_years</t>
+  </si>
+  <si>
+    <t>startup_hardware_engineer_fte</t>
+  </si>
+  <si>
+    <t>Detector and electronics engineer: staffing</t>
+  </si>
+  <si>
+    <t>startup_hardware_engineer_annual</t>
+  </si>
+  <si>
+    <t>Detector and electronics engineer: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>startup_hardware_engineer_years</t>
+  </si>
+  <si>
+    <t>Detector and electronics engineer: funded years</t>
+  </si>
+  <si>
+    <t>startup_hardware_engineer_total</t>
+  </si>
+  <si>
+    <t>Detector and electronics engineer: programme cost</t>
+  </si>
+  <si>
+    <t>startup_hardware_engineer_fte*startup_hardware_engineer_annual*startup_hardware_engineer_years</t>
+  </si>
+  <si>
+    <t>startup_software_fte</t>
+  </si>
+  <si>
+    <t>Software engineers: staffing</t>
+  </si>
+  <si>
+    <t>startup_software_annual</t>
+  </si>
+  <si>
+    <t>Software engineers: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>startup_software_years</t>
+  </si>
+  <si>
+    <t>Software engineers: funded years</t>
+  </si>
+  <si>
+    <t>startup_software_total</t>
+  </si>
+  <si>
+    <t>Software engineers: programme cost</t>
+  </si>
+  <si>
+    <t>startup_software_fte*startup_software_annual*startup_software_years</t>
+  </si>
+  <si>
+    <t>startup_physicist_fte</t>
+  </si>
+  <si>
+    <t>Medical physicist / validation lead: staffing</t>
+  </si>
+  <si>
+    <t>startup_physicist_annual</t>
+  </si>
+  <si>
+    <t>Medical physicist / validation lead: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>startup_physicist_years</t>
+  </si>
+  <si>
+    <t>Medical physicist / validation lead: funded years</t>
+  </si>
+  <si>
+    <t>startup_physicist_total</t>
+  </si>
+  <si>
+    <t>Medical physicist / validation lead: programme cost</t>
+  </si>
+  <si>
+    <t>startup_physicist_fte*startup_physicist_annual*startup_physicist_years</t>
+  </si>
+  <si>
+    <t>startup_technician_fte</t>
+  </si>
+  <si>
+    <t>Assembly and laboratory technician: staffing</t>
+  </si>
+  <si>
+    <t>startup_technician_annual</t>
+  </si>
+  <si>
+    <t>Assembly and laboratory technician: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>startup_technician_years</t>
+  </si>
+  <si>
+    <t>Assembly and laboratory technician: funded years</t>
+  </si>
+  <si>
+    <t>Independent duration; review when changing programme length.</t>
+  </si>
+  <si>
+    <t>startup_technician_total</t>
+  </si>
+  <si>
+    <t>Assembly and laboratory technician: programme cost</t>
+  </si>
+  <si>
+    <t>startup_technician_fte*startup_technician_annual*startup_technician_years</t>
+  </si>
+  <si>
+    <t>startup_quality_fte</t>
+  </si>
+  <si>
+    <t>Quality and regulatory lead: staffing</t>
+  </si>
+  <si>
+    <t>Removed from reduced budget by user; zero retained for editable formulas.</t>
+  </si>
+  <si>
+    <t>startup_quality_annual</t>
+  </si>
+  <si>
+    <t>Quality and regulatory lead: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>startup_quality_years</t>
+  </si>
+  <si>
+    <t>Quality and regulatory lead: funded years</t>
+  </si>
+  <si>
+    <t>startup_quality_total</t>
+  </si>
+  <si>
+    <t>Quality and regulatory lead: programme cost</t>
+  </si>
+  <si>
+    <t>startup_quality_fte*startup_quality_annual*startup_quality_years</t>
+  </si>
+  <si>
+    <t>startup_monitor_fte</t>
+  </si>
+  <si>
+    <t>Clinical monitoring specialist: staffing</t>
+  </si>
+  <si>
+    <t>startup_monitor_annual</t>
+  </si>
+  <si>
+    <t>Clinical monitoring specialist: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>Includes employer contributions. Includes one-shift relief provision.</t>
+  </si>
+  <si>
+    <t>startup_monitor_years</t>
+  </si>
+  <si>
+    <t>Clinical monitoring specialist: funded years</t>
+  </si>
+  <si>
+    <t>startup_monitor_total</t>
+  </si>
+  <si>
+    <t>Clinical monitoring specialist: programme cost</t>
+  </si>
+  <si>
+    <t>startup_monitor_fte*startup_monitor_annual*startup_monitor_years</t>
+  </si>
+  <si>
+    <t>startup_admin_clerk_fte</t>
+  </si>
+  <si>
+    <t>Administrative clerk: staffing</t>
+  </si>
+  <si>
+    <t>startup_admin_clerk_annual</t>
+  </si>
+  <si>
+    <t>Administrative clerk: annual employer cost per FTE</t>
+  </si>
+  <si>
+    <t>User input; total employer cost, consistent with other personnel.</t>
+  </si>
+  <si>
+    <t>startup_admin_clerk_years</t>
+  </si>
+  <si>
+    <t>Administrative clerk: funded years</t>
+  </si>
+  <si>
+    <t>startup_admin_clerk_total</t>
+  </si>
+  <si>
+    <t>Administrative clerk: programme cost</t>
+  </si>
+  <si>
+    <t>startup_admin_clerk_fte*startup_admin_clerk_annual*startup_admin_clerk_years</t>
+  </si>
+  <si>
+    <t>startup_personnel</t>
+  </si>
+  <si>
+    <t>Total personnel</t>
+  </si>
+  <si>
+    <t>startup_ceo_total+startup_architect_total+startup_hardware_engineer_total+startup_software_total+startup_physicist_total+startup_technician_total+startup_quality_total+startup_monitor_total + startup_admin_clerk_total</t>
+  </si>
+  <si>
+    <t>startup_clinical</t>
+  </si>
+  <si>
+    <t>Hospital and clinical programme</t>
+  </si>
+  <si>
+    <t>Reduced to half the previous amount by user.</t>
+  </si>
+  <si>
+    <t>startup_regulatory</t>
+  </si>
+  <si>
+    <t>External regulatory and conformity work</t>
+  </si>
+  <si>
+    <t>startup_space_annual</t>
+  </si>
+  <si>
+    <t>Office and laboratory space: annual cost</t>
+  </si>
+  <si>
+    <t>startup_space_total</t>
+  </si>
+  <si>
+    <t>Office and laboratory space: programme cost</t>
+  </si>
+  <si>
+    <t>startup_space_annual*startup_years</t>
+  </si>
+  <si>
+    <t>startup_it_annual</t>
+  </si>
+  <si>
+    <t>Software tools and IT operations: annual cost</t>
+  </si>
+  <si>
+    <t>startup_it_total</t>
+  </si>
+  <si>
+    <t>Software tools and IT operations: programme cost</t>
+  </si>
+  <si>
+    <t>startup_it_annual*startup_years</t>
+  </si>
+  <si>
+    <t>startup_travel_annual</t>
+  </si>
+  <si>
+    <t>Travel and transport: annual cost</t>
+  </si>
+  <si>
+    <t>startup_travel_total</t>
+  </si>
+  <si>
+    <t>Travel and transport: programme cost</t>
+  </si>
+  <si>
+    <t>startup_travel_annual*startup_years</t>
+  </si>
+  <si>
+    <t>startup_nonhardware</t>
+  </si>
+  <si>
+    <t>Programme expenditure outside hardware package</t>
+  </si>
+  <si>
+    <t>startup_personnel+startup_clinical+startup_regulatory+startup_space_total+startup_it_total+startup_travel_total</t>
+  </si>
+  <si>
+    <t>startup_planned</t>
+  </si>
+  <si>
+    <t>Planned expenditure including first-device contingency</t>
+  </si>
+  <si>
+    <t>startup_hardware_package+startup_nonhardware</t>
+  </si>
+  <si>
+    <t>startup_reserve</t>
+  </si>
+  <si>
+    <t>Programme reserve</t>
+  </si>
+  <si>
+    <t>Fixed allowance: half the previous EUR 504000 reserve; no longer percentage-based.</t>
+  </si>
+  <si>
+    <t>startup_working_capital</t>
+  </si>
+  <si>
+    <t>Working-capital buffer</t>
+  </si>
+  <si>
+    <t>startup_backup</t>
+  </si>
+  <si>
+    <t>Additional backup allowance</t>
+  </si>
+  <si>
+    <t>User-approved allowance bringing the current four-year budget to EUR 4000000; separate from programme reserve.</t>
+  </si>
+  <si>
+    <t>startup_funding</t>
+  </si>
+  <si>
+    <t>Total funding requirement</t>
+  </si>
+  <si>
+    <t>startup_planned+startup_reserve+startup_working_capital+startup_backup</t>
+  </si>
+  <si>
+    <t>startup_rounding</t>
+  </si>
+  <si>
+    <t>Funding display rounding increment</t>
+  </si>
+  <si>
+    <t>startup_funding_rounded</t>
+  </si>
+  <si>
+    <t>Funding requirement rounded up</t>
+  </si>
+  <si>
+    <t>ceil(startup_funding/startup_rounding)*startup_rounding</t>
+  </si>
+  <si>
+    <t>startup_operating</t>
+  </si>
+  <si>
+    <t>Clinical regulatory and operating costs</t>
+  </si>
+  <si>
+    <t>startup_nonhardware-startup_personnel</t>
+  </si>
+  <si>
+    <t>Excludes personnel and reserves.</t>
+  </si>
+  <si>
+    <t>team_ceo_annual</t>
+  </si>
+  <si>
+    <t>ceo annual</t>
+  </si>
+  <si>
+    <t>Linked to costs-reduced.csv.</t>
+  </si>
+  <si>
+    <t>team_ceo_years</t>
+  </si>
+  <si>
+    <t>ceo years</t>
+  </si>
+  <si>
+    <t>team_ceo_total</t>
+  </si>
+  <si>
+    <t>ceo total</t>
+  </si>
+  <si>
+    <t>team_ceo_fte</t>
+  </si>
+  <si>
+    <t>ceo fte</t>
+  </si>
+  <si>
+    <t>team_hardware_engineer_annual</t>
+  </si>
+  <si>
+    <t>hardware engineer annual</t>
+  </si>
+  <si>
+    <t>team_hardware_engineer_years</t>
+  </si>
+  <si>
+    <t>hardware engineer years</t>
+  </si>
+  <si>
+    <t>team_hardware_engineer_total</t>
+  </si>
+  <si>
+    <t>hardware engineer total</t>
+  </si>
+  <si>
+    <t>team_hardware_engineer_fte</t>
+  </si>
+  <si>
+    <t>hardware engineer fte</t>
+  </si>
+  <si>
+    <t>team_software_annual</t>
+  </si>
+  <si>
+    <t>software annual</t>
+  </si>
+  <si>
+    <t>team_software_years</t>
+  </si>
+  <si>
+    <t>software years</t>
+  </si>
+  <si>
+    <t>team_software_total</t>
+  </si>
+  <si>
+    <t>software total</t>
+  </si>
+  <si>
+    <t>team_software_fte</t>
+  </si>
+  <si>
+    <t>software fte</t>
+  </si>
+  <si>
+    <t>team_physicist_annual</t>
+  </si>
+  <si>
+    <t>physicist annual</t>
+  </si>
+  <si>
+    <t>team_physicist_years</t>
+  </si>
+  <si>
+    <t>physicist years</t>
+  </si>
+  <si>
+    <t>team_physicist_total</t>
+  </si>
+  <si>
+    <t>physicist total</t>
+  </si>
+  <si>
+    <t>team_physicist_fte</t>
+  </si>
+  <si>
+    <t>physicist fte</t>
+  </si>
+  <si>
+    <t>team_technician_annual</t>
+  </si>
+  <si>
+    <t>technician annual</t>
+  </si>
+  <si>
+    <t>team_technician_years</t>
+  </si>
+  <si>
+    <t>technician years</t>
+  </si>
+  <si>
+    <t>team_technician_total</t>
+  </si>
+  <si>
+    <t>technician total</t>
+  </si>
+  <si>
+    <t>team_technician_fte</t>
+  </si>
+  <si>
+    <t>technician fte</t>
+  </si>
+  <si>
+    <t>team_admin_clerk_annual</t>
+  </si>
+  <si>
+    <t>admin clerk annual</t>
+  </si>
+  <si>
+    <t>team_admin_clerk_years</t>
+  </si>
+  <si>
+    <t>admin clerk years</t>
+  </si>
+  <si>
+    <t>team_admin_clerk_total</t>
+  </si>
+  <si>
+    <t>admin clerk total</t>
+  </si>
+  <si>
+    <t>team_admin_clerk_fte</t>
+  </si>
+  <si>
+    <t>admin clerk fte</t>
+  </si>
+  <si>
+    <t>team_total</t>
+  </si>
+  <si>
+    <t>programme_pet</t>
+  </si>
+  <si>
+    <t>pet</t>
+  </si>
+  <si>
+    <t>programme_camera</t>
+  </si>
+  <si>
+    <t>camera</t>
+  </si>
+  <si>
+    <t>programme_other_hardware</t>
+  </si>
+  <si>
+    <t>other hardware</t>
+  </si>
+  <si>
+    <t>programme_external_work</t>
+  </si>
+  <si>
+    <t>external work</t>
+  </si>
+  <si>
+    <t>programme_device_reserve</t>
+  </si>
+  <si>
+    <t>device reserve</t>
+  </si>
+  <si>
+    <t>programme_hardware_package</t>
+  </si>
+  <si>
+    <t>hardware package</t>
+  </si>
+  <si>
+    <t>programme_clinical</t>
+  </si>
+  <si>
+    <t>clinical</t>
+  </si>
+  <si>
+    <t>programme_regulatory</t>
+  </si>
+  <si>
+    <t>regulatory</t>
+  </si>
+  <si>
+    <t>programme_first</t>
+  </si>
+  <si>
+    <t>Design year</t>
+  </si>
+  <si>
+    <t>Relative to programme start.</t>
+  </si>
+  <si>
+    <t>programme_second</t>
+  </si>
+  <si>
+    <t>Prototype year</t>
+  </si>
+  <si>
+    <t>programme_clinical_start</t>
+  </si>
+  <si>
+    <t>Clinical phase first year</t>
+  </si>
+  <si>
+    <t>programme_end</t>
+  </si>
+  <si>
+    <t>Programme end</t>
+  </si>
+  <si>
+    <t>programme_pet_count</t>
+  </si>
+  <si>
+    <t>PET demonstrators</t>
+  </si>
+  <si>
+    <t>devices</t>
+  </si>
+  <si>
+    <t>programme_camera_count</t>
+  </si>
+  <si>
+    <t>Compton camera demonstrators</t>
   </si>
 </sst>
 </file>
@@ -1214,6 +1925,54 @@
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="model_argos_market" displayName="model_argos_market" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Item"/>
+    <tableColumn id="3" name="Kind"/>
+    <tableColumn id="4" name="Value"/>
+    <tableColumn id="5" name="Unit"/>
+    <tableColumn id="6" name="Calculation"/>
+    <tableColumn id="7" name="Assumption / source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="model_costs_reduced" displayName="model_costs_reduced" ref="A1:G63" totalsRowShown="0">
+  <autoFilter ref="A1:G63"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Item"/>
+    <tableColumn id="3" name="Kind"/>
+    <tableColumn id="4" name="Value"/>
+    <tableColumn id="5" name="Unit"/>
+    <tableColumn id="6" name="Calculation"/>
+    <tableColumn id="7" name="Assumption / source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="model_startup_team" displayName="model_startup_team" ref="A1:G26" totalsRowShown="0">
+  <autoFilter ref="A1:G26"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Item"/>
+    <tableColumn id="3" name="Kind"/>
+    <tableColumn id="4" name="Value"/>
+    <tableColumn id="5" name="Unit"/>
+    <tableColumn id="6" name="Calculation"/>
+    <tableColumn id="7" name="Assumption / source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="model_startup_programme" displayName="model_startup_programme" ref="A1:G15" totalsRowShown="0">
+  <autoFilter ref="A1:G15"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -4125,4 +4884,2277 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G63"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="57.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="57.7109375" customWidth="1"/>
+    <col min="7" max="7" width="100.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>350</v>
+      </c>
+      <c r="B2" t="s">
+        <v>351</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>352</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1">
+        <v>740000</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>353</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>354</v>
+      </c>
+      <c r="B5" t="s">
+        <v>355</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>357</v>
+      </c>
+      <c r="B6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <f>(('costs-reduced'!D3+'costs-reduced'!D4)+'costs-reduced'!D5)</f>
+        <v>940000.0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B7" t="s">
+        <v>361</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1">
+        <v>200000</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>363</v>
+      </c>
+      <c r="B8" t="s">
+        <v>364</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="1">
+        <v>300000</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>366</v>
+      </c>
+      <c r="B9" t="s">
+        <v>367</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <f>(('costs-reduced'!D6+'costs-reduced'!D7)+'costs-reduced'!D8)</f>
+        <v>1440000.0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B10" t="s">
+        <v>370</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>372</v>
+      </c>
+      <c r="B11" t="s">
+        <v>373</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E11" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B12" t="s">
+        <v>375</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>253</v>
+      </c>
+      <c r="F12" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>376</v>
+      </c>
+      <c r="B13" t="s">
+        <v>377</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2">
+        <f>(('costs-reduced'!D10*'costs-reduced'!D11)*'costs-reduced'!D12)</f>
+        <v>400000.0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>379</v>
+      </c>
+      <c r="B14" t="s">
+        <v>380</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>371</v>
+      </c>
+      <c r="G14" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>382</v>
+      </c>
+      <c r="B15" t="s">
+        <v>383</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>385</v>
+      </c>
+      <c r="B16" t="s">
+        <v>386</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E16" t="s">
+        <v>253</v>
+      </c>
+      <c r="F16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>387</v>
+      </c>
+      <c r="B17" t="s">
+        <v>388</v>
+      </c>
+      <c r="C17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2">
+        <f>(('costs-reduced'!D14*'costs-reduced'!D15)*'costs-reduced'!D16)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>390</v>
+      </c>
+      <c r="B18" t="s">
+        <v>391</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>392</v>
+      </c>
+      <c r="B19" t="s">
+        <v>393</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="1">
+        <v>85000</v>
+      </c>
+      <c r="E19" t="s">
+        <v>87</v>
+      </c>
+      <c r="G19" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>394</v>
+      </c>
+      <c r="B20" t="s">
+        <v>395</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>253</v>
+      </c>
+      <c r="F20" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>396</v>
+      </c>
+      <c r="B21" t="s">
+        <v>397</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="2">
+        <f>(('costs-reduced'!D18*'costs-reduced'!D19)*'costs-reduced'!D20)</f>
+        <v>340000.0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>399</v>
+      </c>
+      <c r="B22" t="s">
+        <v>400</v>
+      </c>
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>371</v>
+      </c>
+      <c r="G22" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>401</v>
+      </c>
+      <c r="B23" t="s">
+        <v>402</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="1">
+        <v>85000</v>
+      </c>
+      <c r="E23" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>403</v>
+      </c>
+      <c r="B24" t="s">
+        <v>404</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>253</v>
+      </c>
+      <c r="F24" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>405</v>
+      </c>
+      <c r="B25" t="s">
+        <v>406</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2">
+        <f>(('costs-reduced'!D22*'costs-reduced'!D23)*'costs-reduced'!D24)</f>
+        <v>340000.0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>408</v>
+      </c>
+      <c r="B26" t="s">
+        <v>409</v>
+      </c>
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="1">
+        <v>1</v>
+      </c>
+      <c r="E26" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>410</v>
+      </c>
+      <c r="B27" t="s">
+        <v>411</v>
+      </c>
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="1">
+        <v>85000</v>
+      </c>
+      <c r="E27" t="s">
+        <v>87</v>
+      </c>
+      <c r="G27" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>412</v>
+      </c>
+      <c r="B28" t="s">
+        <v>413</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>253</v>
+      </c>
+      <c r="F28" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>414</v>
+      </c>
+      <c r="B29" t="s">
+        <v>415</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="2">
+        <f>(('costs-reduced'!D26*'costs-reduced'!D27)*'costs-reduced'!D28)</f>
+        <v>340000.0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>417</v>
+      </c>
+      <c r="B30" t="s">
+        <v>418</v>
+      </c>
+      <c r="C30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="1">
+        <v>1</v>
+      </c>
+      <c r="E30" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>419</v>
+      </c>
+      <c r="B31" t="s">
+        <v>420</v>
+      </c>
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="1">
+        <v>50000</v>
+      </c>
+      <c r="E31" t="s">
+        <v>87</v>
+      </c>
+      <c r="G31" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>421</v>
+      </c>
+      <c r="B32" t="s">
+        <v>422</v>
+      </c>
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="1">
+        <v>3</v>
+      </c>
+      <c r="E32" t="s">
+        <v>253</v>
+      </c>
+      <c r="G32" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
+        <v>424</v>
+      </c>
+      <c r="B33" t="s">
+        <v>425</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="2">
+        <f>(('costs-reduced'!D30*'costs-reduced'!D31)*'costs-reduced'!D32)</f>
+        <v>150000.0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
+        <v>427</v>
+      </c>
+      <c r="B34" t="s">
+        <v>428</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="1">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>371</v>
+      </c>
+      <c r="G34" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>430</v>
+      </c>
+      <c r="B35" t="s">
+        <v>431</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="1">
+        <v>90000</v>
+      </c>
+      <c r="E35" t="s">
+        <v>87</v>
+      </c>
+      <c r="G35" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" t="s">
+        <v>432</v>
+      </c>
+      <c r="B36" t="s">
+        <v>433</v>
+      </c>
+      <c r="C36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E36" t="s">
+        <v>253</v>
+      </c>
+      <c r="F36" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" t="s">
+        <v>434</v>
+      </c>
+      <c r="B37" t="s">
+        <v>435</v>
+      </c>
+      <c r="C37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="2">
+        <f>(('costs-reduced'!D34*'costs-reduced'!D35)*'costs-reduced'!D36)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" t="s">
+        <v>437</v>
+      </c>
+      <c r="B38" t="s">
+        <v>438</v>
+      </c>
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>371</v>
+      </c>
+      <c r="G38" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>439</v>
+      </c>
+      <c r="B39" t="s">
+        <v>440</v>
+      </c>
+      <c r="C39" t="s">
+        <v>9</v>
+      </c>
+      <c r="D39" s="1">
+        <v>80000</v>
+      </c>
+      <c r="E39" t="s">
+        <v>87</v>
+      </c>
+      <c r="G39" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" t="s">
+        <v>442</v>
+      </c>
+      <c r="B40" t="s">
+        <v>443</v>
+      </c>
+      <c r="C40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="1">
+        <v>2</v>
+      </c>
+      <c r="E40" t="s">
+        <v>253</v>
+      </c>
+      <c r="G40" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" t="s">
+        <v>444</v>
+      </c>
+      <c r="B41" t="s">
+        <v>445</v>
+      </c>
+      <c r="C41" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" s="2">
+        <f>(('costs-reduced'!D38*'costs-reduced'!D39)*'costs-reduced'!D40)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" t="s">
+        <v>447</v>
+      </c>
+      <c r="B42" t="s">
+        <v>448</v>
+      </c>
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="1">
+        <v>1</v>
+      </c>
+      <c r="E42" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" t="s">
+        <v>449</v>
+      </c>
+      <c r="B43" t="s">
+        <v>450</v>
+      </c>
+      <c r="C43" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="1">
+        <v>40000</v>
+      </c>
+      <c r="E43" t="s">
+        <v>87</v>
+      </c>
+      <c r="G43" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
+        <v>452</v>
+      </c>
+      <c r="B44" t="s">
+        <v>453</v>
+      </c>
+      <c r="C44" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E44" t="s">
+        <v>253</v>
+      </c>
+      <c r="F44" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" t="s">
+        <v>454</v>
+      </c>
+      <c r="B45" t="s">
+        <v>455</v>
+      </c>
+      <c r="C45" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="2">
+        <f>(('costs-reduced'!D42*'costs-reduced'!D43)*'costs-reduced'!D44)</f>
+        <v>160000.0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" t="s">
+        <v>457</v>
+      </c>
+      <c r="B46" t="s">
+        <v>458</v>
+      </c>
+      <c r="C46" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="2">
+        <f>(((((((('costs-reduced'!D13+'costs-reduced'!D17)+'costs-reduced'!D21)+'costs-reduced'!D25)+'costs-reduced'!D29)+'costs-reduced'!D33)+'costs-reduced'!D37)+'costs-reduced'!D41)+'costs-reduced'!D45)</f>
+        <v>1730000.0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" t="s">
+        <v>460</v>
+      </c>
+      <c r="B47" t="s">
+        <v>461</v>
+      </c>
+      <c r="C47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" s="1">
+        <v>50000</v>
+      </c>
+      <c r="E47" t="s">
+        <v>10</v>
+      </c>
+      <c r="G47" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" t="s">
+        <v>463</v>
+      </c>
+      <c r="B48" t="s">
+        <v>464</v>
+      </c>
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" s="1">
+        <v>25000</v>
+      </c>
+      <c r="E48" t="s">
+        <v>10</v>
+      </c>
+      <c r="G48" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" t="s">
+        <v>465</v>
+      </c>
+      <c r="B49" t="s">
+        <v>466</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="1">
+        <v>10000</v>
+      </c>
+      <c r="E49" t="s">
+        <v>87</v>
+      </c>
+      <c r="G49" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" t="s">
+        <v>467</v>
+      </c>
+      <c r="B50" t="s">
+        <v>468</v>
+      </c>
+      <c r="C50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D50" s="2">
+        <f>('costs-reduced'!D49*'costs-reduced'!D2)</f>
+        <v>40000.0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" t="s">
+        <v>470</v>
+      </c>
+      <c r="B51" t="s">
+        <v>471</v>
+      </c>
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" s="1">
+        <v>20000</v>
+      </c>
+      <c r="E51" t="s">
+        <v>87</v>
+      </c>
+      <c r="G51" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" t="s">
+        <v>472</v>
+      </c>
+      <c r="B52" t="s">
+        <v>473</v>
+      </c>
+      <c r="C52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D52" s="2">
+        <f>('costs-reduced'!D51*'costs-reduced'!D2)</f>
+        <v>80000.0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" t="s">
+        <v>475</v>
+      </c>
+      <c r="B53" t="s">
+        <v>476</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" s="1">
+        <v>30000</v>
+      </c>
+      <c r="E53" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" t="s">
+        <v>477</v>
+      </c>
+      <c r="B54" t="s">
+        <v>478</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54" s="2">
+        <f>('costs-reduced'!D53*'costs-reduced'!D2)</f>
+        <v>120000.0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" t="s">
+        <v>480</v>
+      </c>
+      <c r="B55" t="s">
+        <v>481</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55" s="2">
+        <f>((((('costs-reduced'!D46+'costs-reduced'!D47)+'costs-reduced'!D48)+'costs-reduced'!D50)+'costs-reduced'!D52)+'costs-reduced'!D54)</f>
+        <v>2045000.0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" t="s">
+        <v>483</v>
+      </c>
+      <c r="B56" t="s">
+        <v>484</v>
+      </c>
+      <c r="C56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="2">
+        <f>('costs-reduced'!D9+'costs-reduced'!D55)</f>
+        <v>3485000.0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" t="s">
+        <v>486</v>
+      </c>
+      <c r="B57" t="s">
+        <v>487</v>
+      </c>
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" s="1">
+        <v>252000</v>
+      </c>
+      <c r="E57" t="s">
+        <v>10</v>
+      </c>
+      <c r="G57" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" t="s">
+        <v>489</v>
+      </c>
+      <c r="B58" t="s">
+        <v>490</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" s="1">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>10</v>
+      </c>
+      <c r="G58" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" t="s">
+        <v>491</v>
+      </c>
+      <c r="B59" t="s">
+        <v>492</v>
+      </c>
+      <c r="C59" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" s="1">
+        <v>263000</v>
+      </c>
+      <c r="E59" t="s">
+        <v>10</v>
+      </c>
+      <c r="G59" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" t="s">
+        <v>494</v>
+      </c>
+      <c r="B60" t="s">
+        <v>495</v>
+      </c>
+      <c r="C60" t="s">
+        <v>20</v>
+      </c>
+      <c r="D60" s="2">
+        <f>((('costs-reduced'!D56+'costs-reduced'!D57)+'costs-reduced'!D58)+'costs-reduced'!D59)</f>
+        <v>4000000.0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" t="s">
+        <v>497</v>
+      </c>
+      <c r="B61" t="s">
+        <v>498</v>
+      </c>
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E61" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62" t="s">
+        <v>499</v>
+      </c>
+      <c r="B62" t="s">
+        <v>500</v>
+      </c>
+      <c r="C62" t="s">
+        <v>20</v>
+      </c>
+      <c r="D62" s="2">
+        <f>(CEILING(('costs-reduced'!D60/'costs-reduced'!D61),1)*'costs-reduced'!D61)</f>
+        <v>4000000.0</v>
+      </c>
+      <c r="E62" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63" t="s">
+        <v>502</v>
+      </c>
+      <c r="B63" t="s">
+        <v>503</v>
+      </c>
+      <c r="C63" t="s">
+        <v>20</v>
+      </c>
+      <c r="D63" s="2">
+        <f>('costs-reduced'!D55-'costs-reduced'!D46)</f>
+        <v>315000.0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" t="s">
+        <v>504</v>
+      </c>
+      <c r="G63" t="s">
+        <v>505</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="57.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="57.7109375" customWidth="1"/>
+    <col min="7" max="7" width="100.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2">
+        <f>'costs-reduced'!D11</f>
+        <v>100000.0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G2" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B3" t="s">
+        <v>510</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2">
+        <f>'costs-reduced'!D12</f>
+        <v>4.0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F3" t="s">
+        <v>374</v>
+      </c>
+      <c r="G3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>511</v>
+      </c>
+      <c r="B4" t="s">
+        <v>512</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2">
+        <f>'costs-reduced'!D13</f>
+        <v>400000.0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>376</v>
+      </c>
+      <c r="G4" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>513</v>
+      </c>
+      <c r="B5" t="s">
+        <v>514</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2">
+        <f>'costs-reduced'!D10</f>
+        <v>1.0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>371</v>
+      </c>
+      <c r="F5" t="s">
+        <v>369</v>
+      </c>
+      <c r="G5" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>515</v>
+      </c>
+      <c r="B6" t="s">
+        <v>516</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <f>'costs-reduced'!D19</f>
+        <v>85000.0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" t="s">
+        <v>392</v>
+      </c>
+      <c r="G6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>517</v>
+      </c>
+      <c r="B7" t="s">
+        <v>518</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <f>'costs-reduced'!D20</f>
+        <v>4.0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>253</v>
+      </c>
+      <c r="F7" t="s">
+        <v>394</v>
+      </c>
+      <c r="G7" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>519</v>
+      </c>
+      <c r="B8" t="s">
+        <v>520</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2">
+        <f>'costs-reduced'!D21</f>
+        <v>340000.0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>396</v>
+      </c>
+      <c r="G8" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>521</v>
+      </c>
+      <c r="B9" t="s">
+        <v>522</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <f>'costs-reduced'!D18</f>
+        <v>1.0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>371</v>
+      </c>
+      <c r="F9" t="s">
+        <v>390</v>
+      </c>
+      <c r="G9" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>523</v>
+      </c>
+      <c r="B10" t="s">
+        <v>524</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="2">
+        <f>'costs-reduced'!D23</f>
+        <v>85000.0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" t="s">
+        <v>401</v>
+      </c>
+      <c r="G10" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>525</v>
+      </c>
+      <c r="B11" t="s">
+        <v>526</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2">
+        <f>'costs-reduced'!D24</f>
+        <v>4.0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>253</v>
+      </c>
+      <c r="F11" t="s">
+        <v>403</v>
+      </c>
+      <c r="G11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>527</v>
+      </c>
+      <c r="B12" t="s">
+        <v>528</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2">
+        <f>'costs-reduced'!D25</f>
+        <v>340000.0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>405</v>
+      </c>
+      <c r="G12" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>529</v>
+      </c>
+      <c r="B13" t="s">
+        <v>530</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2">
+        <f>'costs-reduced'!D22</f>
+        <v>1.0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>371</v>
+      </c>
+      <c r="F13" t="s">
+        <v>399</v>
+      </c>
+      <c r="G13" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>531</v>
+      </c>
+      <c r="B14" t="s">
+        <v>532</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2">
+        <f>'costs-reduced'!D27</f>
+        <v>85000.0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F14" t="s">
+        <v>410</v>
+      </c>
+      <c r="G14" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>533</v>
+      </c>
+      <c r="B15" t="s">
+        <v>534</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="2">
+        <f>'costs-reduced'!D28</f>
+        <v>4.0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>253</v>
+      </c>
+      <c r="F15" t="s">
+        <v>412</v>
+      </c>
+      <c r="G15" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>535</v>
+      </c>
+      <c r="B16" t="s">
+        <v>536</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2">
+        <f>'costs-reduced'!D29</f>
+        <v>340000.0</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" t="s">
+        <v>414</v>
+      </c>
+      <c r="G16" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>537</v>
+      </c>
+      <c r="B17" t="s">
+        <v>538</v>
+      </c>
+      <c r="C17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2">
+        <f>'costs-reduced'!D26</f>
+        <v>1.0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>371</v>
+      </c>
+      <c r="F17" t="s">
+        <v>408</v>
+      </c>
+      <c r="G17" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>539</v>
+      </c>
+      <c r="B18" t="s">
+        <v>540</v>
+      </c>
+      <c r="C18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="2">
+        <f>'costs-reduced'!D31</f>
+        <v>50000.0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>87</v>
+      </c>
+      <c r="F18" t="s">
+        <v>419</v>
+      </c>
+      <c r="G18" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>541</v>
+      </c>
+      <c r="B19" t="s">
+        <v>542</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="2">
+        <f>'costs-reduced'!D32</f>
+        <v>3.0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>253</v>
+      </c>
+      <c r="F19" t="s">
+        <v>421</v>
+      </c>
+      <c r="G19" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>543</v>
+      </c>
+      <c r="B20" t="s">
+        <v>544</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="2">
+        <f>'costs-reduced'!D33</f>
+        <v>150000.0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" t="s">
+        <v>424</v>
+      </c>
+      <c r="G20" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>545</v>
+      </c>
+      <c r="B21" t="s">
+        <v>546</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="2">
+        <f>'costs-reduced'!D30</f>
+        <v>1.0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>371</v>
+      </c>
+      <c r="F21" t="s">
+        <v>417</v>
+      </c>
+      <c r="G21" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>547</v>
+      </c>
+      <c r="B22" t="s">
+        <v>548</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="2">
+        <f>'costs-reduced'!D43</f>
+        <v>40000.0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" t="s">
+        <v>449</v>
+      </c>
+      <c r="G22" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>549</v>
+      </c>
+      <c r="B23" t="s">
+        <v>550</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="2">
+        <f>'costs-reduced'!D44</f>
+        <v>4.0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>253</v>
+      </c>
+      <c r="F23" t="s">
+        <v>452</v>
+      </c>
+      <c r="G23" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>551</v>
+      </c>
+      <c r="B24" t="s">
+        <v>552</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="2">
+        <f>'costs-reduced'!D45</f>
+        <v>160000.0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" t="s">
+        <v>454</v>
+      </c>
+      <c r="G24" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>553</v>
+      </c>
+      <c r="B25" t="s">
+        <v>554</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2">
+        <f>'costs-reduced'!D42</f>
+        <v>1.0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>371</v>
+      </c>
+      <c r="F25" t="s">
+        <v>447</v>
+      </c>
+      <c r="G25" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>555</v>
+      </c>
+      <c r="B26" t="s">
+        <v>458</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="2">
+        <f>'costs-reduced'!D46</f>
+        <v>1730000.0</v>
+      </c>
+      <c r="E26" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>457</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="57.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="57.7109375" customWidth="1"/>
+    <col min="7" max="7" width="100.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>556</v>
+      </c>
+      <c r="B2" t="s">
+        <v>557</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2">
+        <f>'costs-reduced'!D3</f>
+        <v>740000.0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>352</v>
+      </c>
+      <c r="G2" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>558</v>
+      </c>
+      <c r="B3" t="s">
+        <v>559</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2">
+        <f>'costs-reduced'!D4</f>
+        <v>100000.0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>353</v>
+      </c>
+      <c r="G3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>560</v>
+      </c>
+      <c r="B4" t="s">
+        <v>561</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2">
+        <f>'costs-reduced'!D5</f>
+        <v>100000.0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>354</v>
+      </c>
+      <c r="G4" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>562</v>
+      </c>
+      <c r="B5" t="s">
+        <v>563</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2">
+        <f>'costs-reduced'!D7</f>
+        <v>200000.0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>360</v>
+      </c>
+      <c r="G5" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>564</v>
+      </c>
+      <c r="B6" t="s">
+        <v>565</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <f>'costs-reduced'!D8</f>
+        <v>300000.0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>363</v>
+      </c>
+      <c r="G6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>566</v>
+      </c>
+      <c r="B7" t="s">
+        <v>567</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <f>'costs-reduced'!D9</f>
+        <v>1440000.0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>366</v>
+      </c>
+      <c r="G7" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>568</v>
+      </c>
+      <c r="B8" t="s">
+        <v>569</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2">
+        <f>'costs-reduced'!D47</f>
+        <v>50000.0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>460</v>
+      </c>
+      <c r="G8" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>570</v>
+      </c>
+      <c r="B9" t="s">
+        <v>571</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <f>'costs-reduced'!D48</f>
+        <v>25000.0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>463</v>
+      </c>
+      <c r="G9" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>572</v>
+      </c>
+      <c r="B10" t="s">
+        <v>573</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>575</v>
+      </c>
+      <c r="B11" t="s">
+        <v>576</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>577</v>
+      </c>
+      <c r="B12" t="s">
+        <v>578</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="1">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>579</v>
+      </c>
+      <c r="B13" t="s">
+        <v>580</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2">
+        <f>'costs-reduced'!D2</f>
+        <v>4.0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>581</v>
+      </c>
+      <c r="B14" t="s">
+        <v>582</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B15" t="s">
+        <v>585</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>583</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Restructure business block, add funding timeline, per-slide model outputs
Deck: remove the obsolete investment slide and the Gantt roadmap; move
Vision & Mission and The DIPC group; order the business block as
strategy, economics, roadmap, demonstrator, team, funding, exit; name
Onkologikoa and BioGipuzkoa consistently; state the two-phase timeline
(2.5 M public 2027-2028, 4 M private 2029-2032). pbt_argos_v2.tex is
now a plain backup copy of the deck before this restructuring.

Cost model: cryogenic system in the startup hardware package with the
backup allowance reduced to keep the 4 M total; build writes one file
per slide under costs/slides so the deck can interleave them.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LunF6tV69q7Y6sP6GhwFZb
</commit_message>
<xml_diff>
--- a/costs/costs.xlsx
+++ b/costs/costs.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="657">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="662">
   <si>
     <t>ID</t>
   </si>
@@ -1299,6 +1299,15 @@
     <t>startup_camera</t>
   </si>
   <si>
+    <t>startup_cryo</t>
+  </si>
+  <si>
+    <t>Cryogenic system</t>
+  </si>
+  <si>
+    <t>Same cryogenic system as the installed-system model (installation.csv); added 2026-09-14.</t>
+  </si>
+  <si>
     <t>startup_other_hardware</t>
   </si>
   <si>
@@ -1314,7 +1323,7 @@
     <t>Raw hardware total</t>
   </si>
   <si>
-    <t>startup_pet+startup_camera+startup_other_hardware</t>
+    <t>startup_pet+startup_camera+startup_cryo+startup_other_hardware</t>
   </si>
   <si>
     <t>startup_external_work</t>
@@ -1716,7 +1725,7 @@
     <t>Additional backup allowance</t>
   </si>
   <si>
-    <t>User-approved allowance bringing the current four-year budget to EUR 4000000; separate from programme reserve.</t>
+    <t>User-approved allowance bringing the four-year budget to EUR 4000000; reduced from 263000 when the cryogenic system was added to the hardware package (2026-09-14). Separate from programme reserve.</t>
   </si>
   <si>
     <t>startup_funding</t>
@@ -1915,6 +1924,12 @@
   </si>
   <si>
     <t>camera</t>
+  </si>
+  <si>
+    <t>programme_cryo</t>
+  </si>
+  <si>
+    <t>cryogenic system</t>
   </si>
   <si>
     <t>programme_other_hardware</t>
@@ -2152,8 +2167,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="model_costs_reduced" displayName="model_costs_reduced" ref="A1:G63" totalsRowShown="0">
-  <autoFilter ref="A1:G63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="model_costs_reduced" displayName="model_costs_reduced" ref="A1:G64" totalsRowShown="0">
+  <autoFilter ref="A1:G64"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -2184,8 +2199,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="model_startup_programme" displayName="model_startup_programme" ref="A1:G15" totalsRowShown="0">
-  <autoFilter ref="A1:G15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="model_startup_programme" displayName="model_startup_programme" ref="A1:G16" totalsRowShown="0">
+  <autoFilter ref="A1:G16"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -5597,7 +5612,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -5694,7 +5709,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="1">
-        <v>100000</v>
+        <v>160000</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -5711,16 +5726,15 @@
         <v>429</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2">
-        <f>(('costs-reduced'!D3+'costs-reduced'!D4)+'costs-reduced'!D5)</f>
-        <v>940000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D6" s="1">
+        <v>100000</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>430</v>
       </c>
     </row>
@@ -5732,15 +5746,16 @@
         <v>432</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="1">
-        <v>200000</v>
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <f>((('costs-reduced'!D3+'costs-reduced'!D4)+'costs-reduced'!D5)+'costs-reduced'!D6)</f>
+        <v>1100000.0</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
       </c>
-      <c r="G7" t="s">
+      <c r="F7" t="s">
         <v>433</v>
       </c>
     </row>
@@ -5755,7 +5770,7 @@
         <v>9</v>
       </c>
       <c r="D8" s="1">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -5772,16 +5787,15 @@
         <v>438</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="2">
-        <f>(('costs-reduced'!D6+'costs-reduced'!D7)+'costs-reduced'!D8)</f>
-        <v>1440000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D9" s="1">
+        <v>300000</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>439</v>
       </c>
     </row>
@@ -5793,12 +5807,16 @@
         <v>441</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D10" s="2">
+        <f>(('costs-reduced'!D7+'costs-reduced'!D8)+'costs-reduced'!D9)</f>
+        <v>1600000.0</v>
       </c>
       <c r="E10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
         <v>442</v>
       </c>
     </row>
@@ -5813,55 +5831,51 @@
         <v>9</v>
       </c>
       <c r="D11" s="1">
-        <v>100000</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>115</v>
-      </c>
-      <c r="G11" t="s">
-        <v>427</v>
+        <v>445</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B12" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="2">
+        <v>9</v>
+      </c>
+      <c r="D12" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E12" t="s">
+        <v>115</v>
+      </c>
+      <c r="G12" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>448</v>
+      </c>
+      <c r="B13" t="s">
+        <v>449</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E13" t="s">
         <v>227</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>447</v>
-      </c>
-      <c r="B13" t="s">
-        <v>448</v>
-      </c>
-      <c r="C13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="2">
-        <f>(('costs-reduced'!D10*'costs-reduced'!D11)*'costs-reduced'!D12)</f>
-        <v>400000.0</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -5872,15 +5886,16 @@
         <v>451</v>
       </c>
       <c r="C14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="D14" s="2">
+        <f>(('costs-reduced'!D11*'costs-reduced'!D12)*'costs-reduced'!D13)</f>
+        <v>400000.0</v>
       </c>
       <c r="E14" t="s">
-        <v>442</v>
-      </c>
-      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s">
         <v>452</v>
       </c>
     </row>
@@ -5895,10 +5910,10 @@
         <v>9</v>
       </c>
       <c r="D15" s="1">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>445</v>
       </c>
       <c r="G15" t="s">
         <v>455</v>
@@ -5912,38 +5927,37 @@
         <v>457</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="2">
+        <v>9</v>
+      </c>
+      <c r="D16" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E16" t="s">
+        <v>115</v>
+      </c>
+      <c r="G16" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>459</v>
+      </c>
+      <c r="B17" t="s">
+        <v>460</v>
+      </c>
+      <c r="C17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E17" t="s">
         <v>227</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F17" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>458</v>
-      </c>
-      <c r="B17" t="s">
-        <v>459</v>
-      </c>
-      <c r="C17" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="2">
-        <f>(('costs-reduced'!D14*'costs-reduced'!D15)*'costs-reduced'!D16)</f>
-        <v>0.0</v>
-      </c>
-      <c r="E17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -5954,75 +5968,75 @@
         <v>462</v>
       </c>
       <c r="C18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D18" s="2">
+        <f>(('costs-reduced'!D15*'costs-reduced'!D16)*'costs-reduced'!D17)</f>
+        <v>0.0</v>
       </c>
       <c r="E18" t="s">
-        <v>442</v>
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B19" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C19" t="s">
         <v>9</v>
       </c>
       <c r="D19" s="1">
-        <v>85000</v>
+        <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B20" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="2">
+        <v>9</v>
+      </c>
+      <c r="D20" s="1">
+        <v>85000</v>
+      </c>
+      <c r="E20" t="s">
+        <v>115</v>
+      </c>
+      <c r="G20" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>468</v>
+      </c>
+      <c r="B21" t="s">
+        <v>469</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E21" t="s">
         <v>227</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F21" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
-        <v>467</v>
-      </c>
-      <c r="B21" t="s">
-        <v>468</v>
-      </c>
-      <c r="C21" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" s="2">
-        <f>(('costs-reduced'!D18*'costs-reduced'!D19)*'costs-reduced'!D20)</f>
-        <v>340000.0</v>
-      </c>
-      <c r="E21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -6033,78 +6047,78 @@
         <v>471</v>
       </c>
       <c r="C22" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D22" s="2">
+        <f>(('costs-reduced'!D19*'costs-reduced'!D20)*'costs-reduced'!D21)</f>
+        <v>340000.0</v>
       </c>
       <c r="E22" t="s">
-        <v>442</v>
-      </c>
-      <c r="G22" t="s">
-        <v>427</v>
+        <v>10</v>
+      </c>
+      <c r="F22" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="1">
-        <v>85000</v>
+        <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>445</v>
       </c>
       <c r="G23" t="s">
-        <v>455</v>
+        <v>430</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B24" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C24" t="s">
-        <v>20</v>
-      </c>
-      <c r="D24" s="2">
+        <v>9</v>
+      </c>
+      <c r="D24" s="1">
+        <v>85000</v>
+      </c>
+      <c r="E24" t="s">
+        <v>115</v>
+      </c>
+      <c r="G24" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>477</v>
+      </c>
+      <c r="B25" t="s">
+        <v>478</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E25" t="s">
         <v>227</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F25" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" t="s">
-        <v>476</v>
-      </c>
-      <c r="B25" t="s">
-        <v>477</v>
-      </c>
-      <c r="C25" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="2">
-        <f>(('costs-reduced'!D22*'costs-reduced'!D23)*'costs-reduced'!D24)</f>
-        <v>340000.0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -6115,75 +6129,75 @@
         <v>480</v>
       </c>
       <c r="C26" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D26" s="2">
+        <f>(('costs-reduced'!D23*'costs-reduced'!D24)*'costs-reduced'!D25)</f>
+        <v>340000.0</v>
       </c>
       <c r="E26" t="s">
-        <v>442</v>
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B27" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C27" t="s">
         <v>9</v>
       </c>
       <c r="D27" s="1">
-        <v>85000</v>
+        <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>115</v>
-      </c>
-      <c r="G27" t="s">
-        <v>427</v>
+        <v>445</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B28" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C28" t="s">
-        <v>20</v>
-      </c>
-      <c r="D28" s="2">
+        <v>9</v>
+      </c>
+      <c r="D28" s="1">
+        <v>85000</v>
+      </c>
+      <c r="E28" t="s">
+        <v>115</v>
+      </c>
+      <c r="G28" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>486</v>
+      </c>
+      <c r="B29" t="s">
+        <v>487</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" t="s">
         <v>227</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F29" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" t="s">
-        <v>485</v>
-      </c>
-      <c r="B29" t="s">
-        <v>486</v>
-      </c>
-      <c r="C29" t="s">
-        <v>20</v>
-      </c>
-      <c r="D29" s="2">
-        <f>(('costs-reduced'!D26*'costs-reduced'!D27)*'costs-reduced'!D28)</f>
-        <v>340000.0</v>
-      </c>
-      <c r="E29" t="s">
-        <v>10</v>
-      </c>
-      <c r="F29" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -6194,53 +6208,54 @@
         <v>489</v>
       </c>
       <c r="C30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D30" s="2">
+        <f>(('costs-reduced'!D27*'costs-reduced'!D28)*'costs-reduced'!D29)</f>
+        <v>340000.0</v>
       </c>
       <c r="E30" t="s">
-        <v>442</v>
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B31" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C31" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="1">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="E31" t="s">
-        <v>115</v>
-      </c>
-      <c r="G31" t="s">
-        <v>427</v>
+        <v>445</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B32" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C32" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="1">
-        <v>3</v>
+        <v>50000</v>
       </c>
       <c r="E32" t="s">
-        <v>227</v>
+        <v>115</v>
       </c>
       <c r="G32" t="s">
-        <v>494</v>
+        <v>430</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -6251,16 +6266,15 @@
         <v>496</v>
       </c>
       <c r="C33" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="2">
-        <f>(('costs-reduced'!D30*'costs-reduced'!D31)*'costs-reduced'!D32)</f>
-        <v>150000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D33" s="1">
+        <v>3</v>
       </c>
       <c r="E33" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" t="s">
+        <v>227</v>
+      </c>
+      <c r="G33" t="s">
         <v>497</v>
       </c>
     </row>
@@ -6272,15 +6286,16 @@
         <v>499</v>
       </c>
       <c r="C34" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34" s="1">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="D34" s="2">
+        <f>(('costs-reduced'!D31*'costs-reduced'!D32)*'costs-reduced'!D33)</f>
+        <v>150000.0</v>
       </c>
       <c r="E34" t="s">
-        <v>442</v>
-      </c>
-      <c r="G34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
         <v>500</v>
       </c>
     </row>
@@ -6295,55 +6310,54 @@
         <v>9</v>
       </c>
       <c r="D35" s="1">
-        <v>90000</v>
+        <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>115</v>
+        <v>445</v>
       </c>
       <c r="G35" t="s">
-        <v>455</v>
+        <v>503</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B36" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C36" t="s">
-        <v>20</v>
-      </c>
-      <c r="D36" s="2">
+        <v>9</v>
+      </c>
+      <c r="D36" s="1">
+        <v>90000</v>
+      </c>
+      <c r="E36" t="s">
+        <v>115</v>
+      </c>
+      <c r="G36" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" t="s">
+        <v>506</v>
+      </c>
+      <c r="B37" t="s">
+        <v>507</v>
+      </c>
+      <c r="C37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E37" t="s">
         <v>227</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F37" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" t="s">
-        <v>505</v>
-      </c>
-      <c r="B37" t="s">
-        <v>506</v>
-      </c>
-      <c r="C37" t="s">
-        <v>20</v>
-      </c>
-      <c r="D37" s="2">
-        <f>(('costs-reduced'!D34*'costs-reduced'!D35)*'costs-reduced'!D36)</f>
-        <v>0.0</v>
-      </c>
-      <c r="E37" t="s">
-        <v>10</v>
-      </c>
-      <c r="F37" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -6354,36 +6368,37 @@
         <v>509</v>
       </c>
       <c r="C38" t="s">
-        <v>9</v>
-      </c>
-      <c r="D38" s="1">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="D38" s="2">
+        <f>(('costs-reduced'!D35*'costs-reduced'!D36)*'costs-reduced'!D37)</f>
+        <v>0.0</v>
       </c>
       <c r="E38" t="s">
-        <v>442</v>
-      </c>
-      <c r="G38" t="s">
-        <v>500</v>
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B39" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
       </c>
       <c r="D39" s="1">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>115</v>
+        <v>445</v>
       </c>
       <c r="G39" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -6397,34 +6412,33 @@
         <v>9</v>
       </c>
       <c r="D40" s="1">
-        <v>2</v>
+        <v>80000</v>
       </c>
       <c r="E40" t="s">
-        <v>227</v>
+        <v>115</v>
       </c>
       <c r="G40" t="s">
-        <v>494</v>
+        <v>515</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B41" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C41" t="s">
-        <v>20</v>
-      </c>
-      <c r="D41" s="2">
-        <f>(('costs-reduced'!D38*'costs-reduced'!D39)*'costs-reduced'!D40)</f>
-        <v>0.0</v>
+        <v>9</v>
+      </c>
+      <c r="D41" s="1">
+        <v>2</v>
       </c>
       <c r="E41" t="s">
-        <v>10</v>
-      </c>
-      <c r="F41" t="s">
-        <v>517</v>
+        <v>227</v>
+      </c>
+      <c r="G41" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -6435,33 +6449,34 @@
         <v>519</v>
       </c>
       <c r="C42" t="s">
-        <v>9</v>
-      </c>
-      <c r="D42" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D42" s="2">
+        <f>(('costs-reduced'!D39*'costs-reduced'!D40)*'costs-reduced'!D41)</f>
+        <v>0.0</v>
       </c>
       <c r="E42" t="s">
-        <v>442</v>
+        <v>10</v>
+      </c>
+      <c r="F42" t="s">
+        <v>520</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B43" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
       </c>
       <c r="D43" s="1">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>115</v>
-      </c>
-      <c r="G43" t="s">
-        <v>522</v>
+        <v>445</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -6472,38 +6487,37 @@
         <v>524</v>
       </c>
       <c r="C44" t="s">
-        <v>20</v>
-      </c>
-      <c r="D44" s="2">
+        <v>9</v>
+      </c>
+      <c r="D44" s="1">
+        <v>40000</v>
+      </c>
+      <c r="E44" t="s">
+        <v>115</v>
+      </c>
+      <c r="G44" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" t="s">
+        <v>526</v>
+      </c>
+      <c r="B45" t="s">
+        <v>527</v>
+      </c>
+      <c r="C45" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E45" t="s">
         <v>227</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F45" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" t="s">
-        <v>525</v>
-      </c>
-      <c r="B45" t="s">
-        <v>526</v>
-      </c>
-      <c r="C45" t="s">
-        <v>20</v>
-      </c>
-      <c r="D45" s="2">
-        <f>(('costs-reduced'!D42*'costs-reduced'!D43)*'costs-reduced'!D44)</f>
-        <v>160000.0</v>
-      </c>
-      <c r="E45" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -6517,8 +6531,8 @@
         <v>20</v>
       </c>
       <c r="D46" s="2">
-        <f>(((((((('costs-reduced'!D13+'costs-reduced'!D17)+'costs-reduced'!D21)+'costs-reduced'!D25)+'costs-reduced'!D29)+'costs-reduced'!D33)+'costs-reduced'!D37)+'costs-reduced'!D41)+'costs-reduced'!D45)</f>
-        <v>1730000.0</v>
+        <f>(('costs-reduced'!D43*'costs-reduced'!D44)*'costs-reduced'!D45)</f>
+        <v>160000.0</v>
       </c>
       <c r="E46" t="s">
         <v>10</v>
@@ -6535,15 +6549,16 @@
         <v>532</v>
       </c>
       <c r="C47" t="s">
-        <v>9</v>
-      </c>
-      <c r="D47" s="1">
-        <v>50000</v>
+        <v>20</v>
+      </c>
+      <c r="D47" s="2">
+        <f>(((((((('costs-reduced'!D14+'costs-reduced'!D18)+'costs-reduced'!D22)+'costs-reduced'!D26)+'costs-reduced'!D30)+'costs-reduced'!D34)+'costs-reduced'!D38)+'costs-reduced'!D42)+'costs-reduced'!D46)</f>
+        <v>1730000.0</v>
       </c>
       <c r="E47" t="s">
         <v>10</v>
       </c>
-      <c r="G47" t="s">
+      <c r="F47" t="s">
         <v>533</v>
       </c>
     </row>
@@ -6558,54 +6573,53 @@
         <v>9</v>
       </c>
       <c r="D48" s="1">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="E48" t="s">
         <v>10</v>
       </c>
       <c r="G48" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
+        <v>537</v>
+      </c>
+      <c r="B49" t="s">
+        <v>538</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="1">
+        <v>25000</v>
+      </c>
+      <c r="E49" t="s">
+        <v>10</v>
+      </c>
+      <c r="G49" t="s">
         <v>536</v>
-      </c>
-      <c r="B49" t="s">
-        <v>537</v>
-      </c>
-      <c r="C49" t="s">
-        <v>9</v>
-      </c>
-      <c r="D49" s="1">
-        <v>10000</v>
-      </c>
-      <c r="E49" t="s">
-        <v>115</v>
-      </c>
-      <c r="G49" t="s">
-        <v>427</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B50" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C50" t="s">
-        <v>20</v>
-      </c>
-      <c r="D50" s="2">
-        <f>('costs-reduced'!D49*'costs-reduced'!D2)</f>
-        <v>40000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D50" s="1">
+        <v>10000</v>
       </c>
       <c r="E50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F50" t="s">
-        <v>540</v>
+        <v>115</v>
+      </c>
+      <c r="G50" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -6616,37 +6630,37 @@
         <v>542</v>
       </c>
       <c r="C51" t="s">
-        <v>9</v>
-      </c>
-      <c r="D51" s="1">
-        <v>20000</v>
+        <v>20</v>
+      </c>
+      <c r="D51" s="2">
+        <f>('costs-reduced'!D50*'costs-reduced'!D2)</f>
+        <v>40000.0</v>
       </c>
       <c r="E51" t="s">
-        <v>115</v>
-      </c>
-      <c r="G51" t="s">
-        <v>427</v>
+        <v>10</v>
+      </c>
+      <c r="F51" t="s">
+        <v>543</v>
       </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B52" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C52" t="s">
-        <v>20</v>
-      </c>
-      <c r="D52" s="2">
-        <f>('costs-reduced'!D51*'costs-reduced'!D2)</f>
-        <v>80000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D52" s="1">
+        <v>20000</v>
       </c>
       <c r="E52" t="s">
-        <v>10</v>
-      </c>
-      <c r="F52" t="s">
-        <v>545</v>
+        <v>115</v>
+      </c>
+      <c r="G52" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -6657,34 +6671,34 @@
         <v>547</v>
       </c>
       <c r="C53" t="s">
-        <v>9</v>
-      </c>
-      <c r="D53" s="1">
-        <v>30000</v>
+        <v>20</v>
+      </c>
+      <c r="D53" s="2">
+        <f>('costs-reduced'!D52*'costs-reduced'!D2)</f>
+        <v>80000.0</v>
       </c>
       <c r="E53" t="s">
-        <v>115</v>
+        <v>10</v>
+      </c>
+      <c r="F53" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="54" spans="1:7">
       <c r="A54" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B54" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C54" t="s">
-        <v>20</v>
-      </c>
-      <c r="D54" s="2">
-        <f>('costs-reduced'!D53*'costs-reduced'!D2)</f>
-        <v>120000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D54" s="1">
+        <v>30000</v>
       </c>
       <c r="E54" t="s">
-        <v>10</v>
-      </c>
-      <c r="F54" t="s">
-        <v>550</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -6698,8 +6712,8 @@
         <v>20</v>
       </c>
       <c r="D55" s="2">
-        <f>((((('costs-reduced'!D46+'costs-reduced'!D47)+'costs-reduced'!D48)+'costs-reduced'!D50)+'costs-reduced'!D52)+'costs-reduced'!D54)</f>
-        <v>2045000.0</v>
+        <f>('costs-reduced'!D54*'costs-reduced'!D2)</f>
+        <v>120000.0</v>
       </c>
       <c r="E55" t="s">
         <v>10</v>
@@ -6719,8 +6733,8 @@
         <v>20</v>
       </c>
       <c r="D56" s="2">
-        <f>('costs-reduced'!D9+'costs-reduced'!D55)</f>
-        <v>3485000.0</v>
+        <f>((((('costs-reduced'!D47+'costs-reduced'!D48)+'costs-reduced'!D49)+'costs-reduced'!D51)+'costs-reduced'!D53)+'costs-reduced'!D55)</f>
+        <v>2045000.0</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
@@ -6737,15 +6751,16 @@
         <v>558</v>
       </c>
       <c r="C57" t="s">
-        <v>9</v>
-      </c>
-      <c r="D57" s="1">
-        <v>252000</v>
+        <v>20</v>
+      </c>
+      <c r="D57" s="2">
+        <f>('costs-reduced'!D10+'costs-reduced'!D56)</f>
+        <v>3645000.0</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
       </c>
-      <c r="G57" t="s">
+      <c r="F57" t="s">
         <v>559</v>
       </c>
     </row>
@@ -6760,33 +6775,33 @@
         <v>9</v>
       </c>
       <c r="D58" s="1">
-        <v>0</v>
+        <v>252000</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
       </c>
       <c r="G58" t="s">
-        <v>500</v>
+        <v>562</v>
       </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B59" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C59" t="s">
         <v>9</v>
       </c>
       <c r="D59" s="1">
-        <v>263000</v>
+        <v>0</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
       </c>
       <c r="G59" t="s">
-        <v>564</v>
+        <v>503</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -6797,16 +6812,15 @@
         <v>566</v>
       </c>
       <c r="C60" t="s">
-        <v>20</v>
-      </c>
-      <c r="D60" s="2">
-        <f>((('costs-reduced'!D56+'costs-reduced'!D57)+'costs-reduced'!D58)+'costs-reduced'!D59)</f>
-        <v>4000000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D60" s="1">
+        <v>103000</v>
       </c>
       <c r="E60" t="s">
         <v>10</v>
       </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
         <v>567</v>
       </c>
     </row>
@@ -6818,34 +6832,34 @@
         <v>569</v>
       </c>
       <c r="C61" t="s">
-        <v>9</v>
-      </c>
-      <c r="D61" s="1">
-        <v>100000</v>
+        <v>20</v>
+      </c>
+      <c r="D61" s="2">
+        <f>((('costs-reduced'!D57+'costs-reduced'!D58)+'costs-reduced'!D59)+'costs-reduced'!D60)</f>
+        <v>4000000.0</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
       </c>
+      <c r="F61" t="s">
+        <v>570</v>
+      </c>
     </row>
     <row r="62" spans="1:7">
       <c r="A62" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B62" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C62" t="s">
-        <v>20</v>
-      </c>
-      <c r="D62" s="2">
-        <f>(CEILING(('costs-reduced'!D60/'costs-reduced'!D61),1)*'costs-reduced'!D61)</f>
-        <v>4000000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D62" s="1">
+        <v>100000</v>
       </c>
       <c r="E62" t="s">
         <v>10</v>
-      </c>
-      <c r="F62" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -6859,8 +6873,8 @@
         <v>20</v>
       </c>
       <c r="D63" s="2">
-        <f>('costs-reduced'!D55-'costs-reduced'!D46)</f>
-        <v>315000.0</v>
+        <f>(CEILING(('costs-reduced'!D61/'costs-reduced'!D62),1)*'costs-reduced'!D62)</f>
+        <v>4000000.0</v>
       </c>
       <c r="E63" t="s">
         <v>10</v>
@@ -6868,8 +6882,29 @@
       <c r="F63" t="s">
         <v>575</v>
       </c>
-      <c r="G63" t="s">
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64" t="s">
         <v>576</v>
+      </c>
+      <c r="B64" t="s">
+        <v>577</v>
+      </c>
+      <c r="C64" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64" s="2">
+        <f>('costs-reduced'!D56-'costs-reduced'!D47)</f>
+        <v>315000.0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" t="s">
+        <v>578</v>
+      </c>
+      <c r="G64" t="s">
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -6919,599 +6954,599 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B2" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
       </c>
       <c r="D2" s="2">
-        <f>'costs-reduced'!D11</f>
+        <f>'costs-reduced'!D12</f>
         <v>100000.0</v>
       </c>
       <c r="E2" t="s">
         <v>115</v>
       </c>
       <c r="F2" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="G2" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B3" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
       </c>
       <c r="D3" s="2">
-        <f>'costs-reduced'!D12</f>
+        <f>'costs-reduced'!D13</f>
         <v>4.0</v>
       </c>
       <c r="E3" t="s">
         <v>227</v>
       </c>
       <c r="F3" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="G3" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B4" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="2">
-        <f>'costs-reduced'!D13</f>
+        <f>'costs-reduced'!D14</f>
         <v>400000.0</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="G4" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B5" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="2">
-        <f>'costs-reduced'!D10</f>
+        <f>'costs-reduced'!D11</f>
         <v>1.0</v>
       </c>
       <c r="E5" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F5" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="G5" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="B6" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" s="2">
-        <f>'costs-reduced'!D19</f>
+        <f>'costs-reduced'!D20</f>
         <v>85000.0</v>
       </c>
       <c r="E6" t="s">
         <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="G6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="B7" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7" s="2">
-        <f>'costs-reduced'!D20</f>
+        <f>'costs-reduced'!D21</f>
         <v>4.0</v>
       </c>
       <c r="E7" t="s">
         <v>227</v>
       </c>
       <c r="F7" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="G7" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B8" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="2">
-        <f>'costs-reduced'!D21</f>
+        <f>'costs-reduced'!D22</f>
         <v>340000.0</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="G8" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B9" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="2">
-        <f>'costs-reduced'!D18</f>
+        <f>'costs-reduced'!D19</f>
         <v>1.0</v>
       </c>
       <c r="E9" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F9" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G9" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B10" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2">
-        <f>'costs-reduced'!D23</f>
+        <f>'costs-reduced'!D24</f>
         <v>85000.0</v>
       </c>
       <c r="E10" t="s">
         <v>115</v>
       </c>
       <c r="F10" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="G10" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B11" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
       </c>
       <c r="D11" s="2">
-        <f>'costs-reduced'!D24</f>
+        <f>'costs-reduced'!D25</f>
         <v>4.0</v>
       </c>
       <c r="E11" t="s">
         <v>227</v>
       </c>
       <c r="F11" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="G11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B12" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
       </c>
       <c r="D12" s="2">
-        <f>'costs-reduced'!D25</f>
+        <f>'costs-reduced'!D26</f>
         <v>340000.0</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="G12" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B13" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
       </c>
       <c r="D13" s="2">
-        <f>'costs-reduced'!D22</f>
+        <f>'costs-reduced'!D23</f>
         <v>1.0</v>
       </c>
       <c r="E13" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F13" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="G13" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="B14" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="2">
-        <f>'costs-reduced'!D27</f>
+        <f>'costs-reduced'!D28</f>
         <v>85000.0</v>
       </c>
       <c r="E14" t="s">
         <v>115</v>
       </c>
       <c r="F14" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="G14" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="B15" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
       </c>
       <c r="D15" s="2">
-        <f>'costs-reduced'!D28</f>
+        <f>'costs-reduced'!D29</f>
         <v>4.0</v>
       </c>
       <c r="E15" t="s">
         <v>227</v>
       </c>
       <c r="F15" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="G15" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="B16" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="2">
-        <f>'costs-reduced'!D29</f>
+        <f>'costs-reduced'!D30</f>
         <v>340000.0</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G16" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B17" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
       </c>
       <c r="D17" s="2">
-        <f>'costs-reduced'!D26</f>
+        <f>'costs-reduced'!D27</f>
         <v>1.0</v>
       </c>
       <c r="E17" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F17" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="G17" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="B18" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
       </c>
       <c r="D18" s="2">
-        <f>'costs-reduced'!D31</f>
+        <f>'costs-reduced'!D32</f>
         <v>50000.0</v>
       </c>
       <c r="E18" t="s">
         <v>115</v>
       </c>
       <c r="F18" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="G18" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="B19" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="C19" t="s">
         <v>20</v>
       </c>
       <c r="D19" s="2">
-        <f>'costs-reduced'!D32</f>
+        <f>'costs-reduced'!D33</f>
         <v>3.0</v>
       </c>
       <c r="E19" t="s">
         <v>227</v>
       </c>
       <c r="F19" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G19" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="B20" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="C20" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="2">
-        <f>'costs-reduced'!D33</f>
+        <f>'costs-reduced'!D34</f>
         <v>150000.0</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G20" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="B21" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="C21" t="s">
         <v>20</v>
       </c>
       <c r="D21" s="2">
-        <f>'costs-reduced'!D30</f>
+        <f>'costs-reduced'!D31</f>
         <v>1.0</v>
       </c>
       <c r="E21" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F21" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="G21" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="B22" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="C22" t="s">
         <v>20</v>
       </c>
       <c r="D22" s="2">
-        <f>'costs-reduced'!D43</f>
+        <f>'costs-reduced'!D44</f>
         <v>40000.0</v>
       </c>
       <c r="E22" t="s">
         <v>115</v>
       </c>
       <c r="F22" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="G22" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="B23" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
       </c>
       <c r="D23" s="2">
-        <f>'costs-reduced'!D44</f>
+        <f>'costs-reduced'!D45</f>
         <v>4.0</v>
       </c>
       <c r="E23" t="s">
         <v>227</v>
       </c>
       <c r="F23" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="G23" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B24" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="C24" t="s">
         <v>20</v>
       </c>
       <c r="D24" s="2">
-        <f>'costs-reduced'!D45</f>
+        <f>'costs-reduced'!D46</f>
         <v>160000.0</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="G24" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="B25" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="C25" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="2">
-        <f>'costs-reduced'!D42</f>
+        <f>'costs-reduced'!D43</f>
         <v>1.0</v>
       </c>
       <c r="E25" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F25" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="G25" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B26" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="C26" t="s">
         <v>20</v>
       </c>
       <c r="D26" s="2">
-        <f>'costs-reduced'!D46</f>
+        <f>'costs-reduced'!D47</f>
         <v>1730000.0</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -7524,7 +7559,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -7561,10 +7596,10 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="B2" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -7580,15 +7615,15 @@
         <v>422</v>
       </c>
       <c r="G2" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="B3" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -7604,22 +7639,22 @@
         <v>424</v>
       </c>
       <c r="G3" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="B4" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="2">
         <f>'costs-reduced'!D5</f>
-        <v>100000.0</v>
+        <v>160000.0</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -7628,46 +7663,46 @@
         <v>425</v>
       </c>
       <c r="G4" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="B5" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="2">
-        <f>'costs-reduced'!D7</f>
-        <v>200000.0</v>
+        <f>'costs-reduced'!D6</f>
+        <v>100000.0</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="G5" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="B6" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" s="2">
         <f>'costs-reduced'!D8</f>
-        <v>300000.0</v>
+        <v>200000.0</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -7676,22 +7711,22 @@
         <v>434</v>
       </c>
       <c r="G6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="B7" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7" s="2">
         <f>'costs-reduced'!D9</f>
-        <v>1440000.0</v>
+        <v>300000.0</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -7700,46 +7735,46 @@
         <v>437</v>
       </c>
       <c r="G7" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="B8" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="2">
-        <f>'costs-reduced'!D47</f>
-        <v>50000.0</v>
+        <f>'costs-reduced'!D10</f>
+        <v>1600000.0</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>531</v>
+        <v>440</v>
       </c>
       <c r="G8" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="B9" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="2">
         <f>'costs-reduced'!D48</f>
-        <v>25000.0</v>
+        <v>50000.0</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -7748,58 +7783,65 @@
         <v>534</v>
       </c>
       <c r="G9" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="B10" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="D10" s="2">
+        <f>'costs-reduced'!D49</f>
+        <v>25000.0</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>537</v>
       </c>
       <c r="G10" t="s">
-        <v>645</v>
+        <v>582</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="B11" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
         <v>89</v>
       </c>
+      <c r="G11" t="s">
+        <v>650</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B12" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="C12" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" t="s">
         <v>89</v>
@@ -7807,48 +7849,48 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B13" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="2">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>655</v>
+      </c>
+      <c r="B14" t="s">
+        <v>656</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2">
         <f>'costs-reduced'!D2</f>
         <v>4.0</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E14" t="s">
         <v>89</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F14" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>652</v>
-      </c>
-      <c r="B14" t="s">
-        <v>653</v>
-      </c>
-      <c r="C14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B15" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="C15" t="s">
         <v>9</v>
@@ -7857,7 +7899,24 @@
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>654</v>
+        <v>659</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>660</v>
+      </c>
+      <c r="B16" t="s">
+        <v>661</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final deck: second review pass and regulatory budget
Guejo spelling throughout, duplicated Taasti result removed, ARGOS as
the proposed spin-off, sentence-case titles, prospects wording, 2025
centre count in the map caption. External regulatory work raised to
125 k with the backup row removed and the reserve adjusted, keeping the
four-year budget at 4 M.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LunF6tV69q7Y6sP6GhwFZb
</commit_message>
<xml_diff>
--- a/costs/costs.xlsx
+++ b/costs/costs.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="660">
   <si>
     <t>ID</t>
   </si>
@@ -1641,6 +1641,9 @@
     <t>External regulatory and conformity work</t>
   </si>
   <si>
+    <t>Notified-body conformity assessment and external regulatory support; raised from 25000 on 2026-09-15.</t>
+  </si>
+  <si>
     <t>startup_space_annual</t>
   </si>
   <si>
@@ -1710,7 +1713,7 @@
     <t>Programme reserve</t>
   </si>
   <si>
-    <t>Fixed allowance: half the previous EUR 504000 reserve; no longer percentage-based.</t>
+    <t>Fixed allowance; adjusted by +3000 on 2026-09-15 when the backup row was removed, keeping the four-year budget at EUR 4000000.</t>
   </si>
   <si>
     <t>startup_working_capital</t>
@@ -1719,22 +1722,13 @@
     <t>Working-capital buffer</t>
   </si>
   <si>
-    <t>startup_backup</t>
-  </si>
-  <si>
-    <t>Additional backup allowance</t>
-  </si>
-  <si>
-    <t>User-approved allowance bringing the four-year budget to EUR 4000000; reduced from 263000 when the cryogenic system was added to the hardware package (2026-09-14). Separate from programme reserve.</t>
-  </si>
-  <si>
     <t>startup_funding</t>
   </si>
   <si>
     <t>Total funding requirement</t>
   </si>
   <si>
-    <t>startup_planned+startup_reserve+startup_working_capital+startup_backup</t>
+    <t>startup_planned+startup_reserve+startup_working_capital</t>
   </si>
   <si>
     <t>startup_rounding</t>
@@ -2167,8 +2161,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="model_costs_reduced" displayName="model_costs_reduced" ref="A1:G64" totalsRowShown="0">
-  <autoFilter ref="A1:G64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="model_costs_reduced" displayName="model_costs_reduced" ref="A1:G63" totalsRowShown="0">
+  <autoFilter ref="A1:G63"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Item"/>
@@ -5612,7 +5606,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -6593,21 +6587,21 @@
         <v>9</v>
       </c>
       <c r="D49" s="1">
-        <v>25000</v>
+        <v>125000</v>
       </c>
       <c r="E49" t="s">
         <v>10</v>
       </c>
       <c r="G49" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B50" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="C50" t="s">
         <v>9</v>
@@ -6624,10 +6618,10 @@
     </row>
     <row r="51" spans="1:7">
       <c r="A51" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B51" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C51" t="s">
         <v>20</v>
@@ -6640,15 +6634,15 @@
         <v>10</v>
       </c>
       <c r="F51" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B52" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C52" t="s">
         <v>9</v>
@@ -6665,10 +6659,10 @@
     </row>
     <row r="53" spans="1:7">
       <c r="A53" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B53" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C53" t="s">
         <v>20</v>
@@ -6681,15 +6675,15 @@
         <v>10</v>
       </c>
       <c r="F53" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="54" spans="1:7">
       <c r="A54" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B54" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C54" t="s">
         <v>9</v>
@@ -6703,10 +6697,10 @@
     </row>
     <row r="55" spans="1:7">
       <c r="A55" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B55" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C55" t="s">
         <v>20</v>
@@ -6719,77 +6713,77 @@
         <v>10</v>
       </c>
       <c r="F55" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B56" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C56" t="s">
         <v>20</v>
       </c>
       <c r="D56" s="2">
         <f>((((('costs-reduced'!D47+'costs-reduced'!D48)+'costs-reduced'!D49)+'costs-reduced'!D51)+'costs-reduced'!D53)+'costs-reduced'!D55)</f>
-        <v>2045000.0</v>
+        <v>2145000.0</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
       </c>
       <c r="F56" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B57" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C57" t="s">
         <v>20</v>
       </c>
       <c r="D57" s="2">
         <f>('costs-reduced'!D10+'costs-reduced'!D56)</f>
-        <v>3645000.0</v>
+        <v>3745000.0</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
       </c>
       <c r="F57" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B58" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C58" t="s">
         <v>9</v>
       </c>
       <c r="D58" s="1">
-        <v>252000</v>
+        <v>255000</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
       </c>
       <c r="G58" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B59" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C59" t="s">
         <v>9</v>
@@ -6806,43 +6800,40 @@
     </row>
     <row r="60" spans="1:7">
       <c r="A60" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B60" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C60" t="s">
-        <v>9</v>
-      </c>
-      <c r="D60" s="1">
-        <v>103000</v>
+        <v>20</v>
+      </c>
+      <c r="D60" s="2">
+        <f>(('costs-reduced'!D57+'costs-reduced'!D58)+'costs-reduced'!D59)</f>
+        <v>4000000.0</v>
       </c>
       <c r="E60" t="s">
         <v>10</v>
       </c>
-      <c r="G60" t="s">
-        <v>567</v>
+      <c r="F60" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="61" spans="1:7">
       <c r="A61" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B61" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C61" t="s">
-        <v>20</v>
-      </c>
-      <c r="D61" s="2">
-        <f>((('costs-reduced'!D57+'costs-reduced'!D58)+'costs-reduced'!D59)+'costs-reduced'!D60)</f>
-        <v>4000000.0</v>
+        <v>9</v>
+      </c>
+      <c r="D61" s="1">
+        <v>100000</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
-      </c>
-      <c r="F61" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -6853,58 +6844,41 @@
         <v>572</v>
       </c>
       <c r="C62" t="s">
-        <v>9</v>
-      </c>
-      <c r="D62" s="1">
-        <v>100000</v>
+        <v>20</v>
+      </c>
+      <c r="D62" s="2">
+        <f>(CEILING(('costs-reduced'!D60/'costs-reduced'!D61),1)*'costs-reduced'!D61)</f>
+        <v>4000000.0</v>
       </c>
       <c r="E62" t="s">
         <v>10</v>
       </c>
+      <c r="F62" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="63" spans="1:7">
       <c r="A63" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B63" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C63" t="s">
         <v>20</v>
       </c>
       <c r="D63" s="2">
-        <f>(CEILING(('costs-reduced'!D61/'costs-reduced'!D62),1)*'costs-reduced'!D62)</f>
-        <v>4000000.0</v>
+        <f>('costs-reduced'!D56-'costs-reduced'!D47)</f>
+        <v>415000.0</v>
       </c>
       <c r="E63" t="s">
         <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
-      <c r="A64" t="s">
         <v>576</v>
       </c>
-      <c r="B64" t="s">
+      <c r="G63" t="s">
         <v>577</v>
-      </c>
-      <c r="C64" t="s">
-        <v>20</v>
-      </c>
-      <c r="D64" s="2">
-        <f>('costs-reduced'!D56-'costs-reduced'!D47)</f>
-        <v>315000.0</v>
-      </c>
-      <c r="E64" t="s">
-        <v>10</v>
-      </c>
-      <c r="F64" t="s">
-        <v>578</v>
-      </c>
-      <c r="G64" t="s">
-        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -6954,10 +6928,10 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -6973,15 +6947,15 @@
         <v>446</v>
       </c>
       <c r="G2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B3" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -6997,15 +6971,15 @@
         <v>448</v>
       </c>
       <c r="G3" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B4" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
@@ -7021,15 +6995,15 @@
         <v>450</v>
       </c>
       <c r="G4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B5" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -7045,15 +7019,15 @@
         <v>443</v>
       </c>
       <c r="G5" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B6" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
@@ -7069,15 +7043,15 @@
         <v>466</v>
       </c>
       <c r="G6" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B7" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -7093,15 +7067,15 @@
         <v>468</v>
       </c>
       <c r="G7" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B8" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -7117,15 +7091,15 @@
         <v>470</v>
       </c>
       <c r="G8" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B9" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
@@ -7141,15 +7115,15 @@
         <v>464</v>
       </c>
       <c r="G9" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B10" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
@@ -7165,15 +7139,15 @@
         <v>475</v>
       </c>
       <c r="G10" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B11" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
@@ -7189,15 +7163,15 @@
         <v>477</v>
       </c>
       <c r="G11" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B12" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
@@ -7213,15 +7187,15 @@
         <v>479</v>
       </c>
       <c r="G12" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B13" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -7237,15 +7211,15 @@
         <v>473</v>
       </c>
       <c r="G13" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B14" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
@@ -7261,15 +7235,15 @@
         <v>484</v>
       </c>
       <c r="G14" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B15" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -7285,15 +7259,15 @@
         <v>486</v>
       </c>
       <c r="G15" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B16" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
@@ -7309,15 +7283,15 @@
         <v>488</v>
       </c>
       <c r="G16" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B17" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -7333,15 +7307,15 @@
         <v>482</v>
       </c>
       <c r="G17" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B18" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
@@ -7357,15 +7331,15 @@
         <v>493</v>
       </c>
       <c r="G18" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B19" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C19" t="s">
         <v>20</v>
@@ -7381,15 +7355,15 @@
         <v>495</v>
       </c>
       <c r="G19" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B20" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="C20" t="s">
         <v>20</v>
@@ -7405,15 +7379,15 @@
         <v>498</v>
       </c>
       <c r="G20" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B21" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="C21" t="s">
         <v>20</v>
@@ -7429,15 +7403,15 @@
         <v>491</v>
       </c>
       <c r="G21" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="B22" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="C22" t="s">
         <v>20</v>
@@ -7453,15 +7427,15 @@
         <v>523</v>
       </c>
       <c r="G22" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B23" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
@@ -7477,15 +7451,15 @@
         <v>526</v>
       </c>
       <c r="G23" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B24" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="C24" t="s">
         <v>20</v>
@@ -7501,15 +7475,15 @@
         <v>528</v>
       </c>
       <c r="G24" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="B25" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="C25" t="s">
         <v>20</v>
@@ -7525,12 +7499,12 @@
         <v>521</v>
       </c>
       <c r="G25" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="B26" t="s">
         <v>532</v>
@@ -7596,10 +7570,10 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B2" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -7615,15 +7589,15 @@
         <v>422</v>
       </c>
       <c r="G2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B3" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -7639,15 +7613,15 @@
         <v>424</v>
       </c>
       <c r="G3" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B4" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
@@ -7663,15 +7637,15 @@
         <v>425</v>
       </c>
       <c r="G4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B5" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -7687,15 +7661,15 @@
         <v>428</v>
       </c>
       <c r="G5" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B6" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
@@ -7711,15 +7685,15 @@
         <v>434</v>
       </c>
       <c r="G6" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B7" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -7735,15 +7709,15 @@
         <v>437</v>
       </c>
       <c r="G7" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B8" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -7759,15 +7733,15 @@
         <v>440</v>
       </c>
       <c r="G8" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B9" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
@@ -7783,22 +7757,22 @@
         <v>534</v>
       </c>
       <c r="G9" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B10" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2">
         <f>'costs-reduced'!D49</f>
-        <v>25000.0</v>
+        <v>125000.0</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -7807,15 +7781,15 @@
         <v>537</v>
       </c>
       <c r="G10" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="B11" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -7827,15 +7801,15 @@
         <v>89</v>
       </c>
       <c r="G11" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B12" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="C12" t="s">
         <v>9</v>
@@ -7849,10 +7823,10 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B13" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
@@ -7866,10 +7840,10 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="B14" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
@@ -7887,10 +7861,10 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B15" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C15" t="s">
         <v>9</v>
@@ -7899,15 +7873,15 @@
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B16" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C16" t="s">
         <v>9</v>
@@ -7916,7 +7890,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>